<commit_message>
Halloween check-in: groep compleet, baannummer pas bij aankomst, tekst tweede bevestiging
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/events/2026-halloween-padel/checkin/halloween-checkin-lijst.xlsx
+++ b/events/2026-halloween-padel/checkin/halloween-checkin-lijst.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Uitleg check-in" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Check-in'!$A$4:$N$404</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Check-in'!$A$4:$O$404</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N404"/>
+  <dimension ref="A1:O404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -545,6 +545,7 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="26" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -566,7 +567,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Geel = vult Lars in na de boeking (baannummer). Blauw = vult de check-in in op de dag. Wit = komt uit de betaling. Grijs = voorbeeld, mag weg.</t>
+          <t>Geel = vult Lars in na de boeking (baannummer, de spelers horen dit pas bij de check-in). Blauw = vult de check-in in op de dag. Wit = komt uit de betaling. Grijs = voorbeeld, mag weg.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -648,6 +649,11 @@
       <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Mollie-betaling</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>Groep compleet</t>
         </is>
       </c>
     </row>
@@ -709,6 +715,10 @@
           <t>tr_voorbeeld</t>
         </is>
       </c>
+      <c r="O5" s="6">
+        <f>IF(D5="","",IF(COUNTIFS($A$5:$A$404,A5,$D$5:$D$404,D5,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A5,$D$5:$D$404,D5,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -768,6 +778,10 @@
           <t>tr_voorbeeld</t>
         </is>
       </c>
+      <c r="O6" s="6">
+        <f>IF(D6="","",IF(COUNTIFS($A$5:$A$404,A6,$D$5:$D$404,D6,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A6,$D$5:$D$404,D6,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -835,6 +849,10 @@
           <t>tr_voorbeeld</t>
         </is>
       </c>
+      <c r="O7" s="6">
+        <f>IF(D7="","",IF(COUNTIFS($A$5:$A$404,A7,$D$5:$D$404,D7,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A7,$D$5:$D$404,D7,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -897,6 +915,10 @@
         <is>
           <t>tr_voorbeeld</t>
         </is>
+      </c>
+      <c r="O8" s="6">
+        <f>IF(D8="","",IF(COUNTIFS($A$5:$A$404,A8,$D$5:$D$404,D8,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A8,$D$5:$D$404,D8,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -917,6 +939,10 @@
       <c r="L9" s="9" t="n"/>
       <c r="M9" s="9" t="n"/>
       <c r="N9" s="11" t="n"/>
+      <c r="O9" s="11">
+        <f>IF(D9="","",IF(COUNTIFS($A$5:$A$404,A9,$D$5:$D$404,D9,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A9,$D$5:$D$404,D9,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="n"/>
@@ -936,6 +962,10 @@
       <c r="L10" s="9" t="n"/>
       <c r="M10" s="9" t="n"/>
       <c r="N10" s="11" t="n"/>
+      <c r="O10" s="11">
+        <f>IF(D10="","",IF(COUNTIFS($A$5:$A$404,A10,$D$5:$D$404,D10,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A10,$D$5:$D$404,D10,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="n"/>
@@ -955,6 +985,10 @@
       <c r="L11" s="9" t="n"/>
       <c r="M11" s="9" t="n"/>
       <c r="N11" s="11" t="n"/>
+      <c r="O11" s="11">
+        <f>IF(D11="","",IF(COUNTIFS($A$5:$A$404,A11,$D$5:$D$404,D11,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A11,$D$5:$D$404,D11,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="n"/>
@@ -974,6 +1008,10 @@
       <c r="L12" s="9" t="n"/>
       <c r="M12" s="9" t="n"/>
       <c r="N12" s="11" t="n"/>
+      <c r="O12" s="11">
+        <f>IF(D12="","",IF(COUNTIFS($A$5:$A$404,A12,$D$5:$D$404,D12,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A12,$D$5:$D$404,D12,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="n"/>
@@ -993,6 +1031,10 @@
       <c r="L13" s="9" t="n"/>
       <c r="M13" s="9" t="n"/>
       <c r="N13" s="11" t="n"/>
+      <c r="O13" s="11">
+        <f>IF(D13="","",IF(COUNTIFS($A$5:$A$404,A13,$D$5:$D$404,D13,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A13,$D$5:$D$404,D13,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="n"/>
@@ -1012,6 +1054,10 @@
       <c r="L14" s="9" t="n"/>
       <c r="M14" s="9" t="n"/>
       <c r="N14" s="11" t="n"/>
+      <c r="O14" s="11">
+        <f>IF(D14="","",IF(COUNTIFS($A$5:$A$404,A14,$D$5:$D$404,D14,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A14,$D$5:$D$404,D14,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="n"/>
@@ -1031,6 +1077,10 @@
       <c r="L15" s="9" t="n"/>
       <c r="M15" s="9" t="n"/>
       <c r="N15" s="11" t="n"/>
+      <c r="O15" s="11">
+        <f>IF(D15="","",IF(COUNTIFS($A$5:$A$404,A15,$D$5:$D$404,D15,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A15,$D$5:$D$404,D15,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="n"/>
@@ -1050,6 +1100,10 @@
       <c r="L16" s="9" t="n"/>
       <c r="M16" s="9" t="n"/>
       <c r="N16" s="11" t="n"/>
+      <c r="O16" s="11">
+        <f>IF(D16="","",IF(COUNTIFS($A$5:$A$404,A16,$D$5:$D$404,D16,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A16,$D$5:$D$404,D16,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="n"/>
@@ -1069,6 +1123,10 @@
       <c r="L17" s="9" t="n"/>
       <c r="M17" s="9" t="n"/>
       <c r="N17" s="11" t="n"/>
+      <c r="O17" s="11">
+        <f>IF(D17="","",IF(COUNTIFS($A$5:$A$404,A17,$D$5:$D$404,D17,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A17,$D$5:$D$404,D17,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="n"/>
@@ -1088,6 +1146,10 @@
       <c r="L18" s="9" t="n"/>
       <c r="M18" s="9" t="n"/>
       <c r="N18" s="11" t="n"/>
+      <c r="O18" s="11">
+        <f>IF(D18="","",IF(COUNTIFS($A$5:$A$404,A18,$D$5:$D$404,D18,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A18,$D$5:$D$404,D18,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="n"/>
@@ -1107,6 +1169,10 @@
       <c r="L19" s="9" t="n"/>
       <c r="M19" s="9" t="n"/>
       <c r="N19" s="11" t="n"/>
+      <c r="O19" s="11">
+        <f>IF(D19="","",IF(COUNTIFS($A$5:$A$404,A19,$D$5:$D$404,D19,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A19,$D$5:$D$404,D19,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="n"/>
@@ -1126,6 +1192,10 @@
       <c r="L20" s="9" t="n"/>
       <c r="M20" s="9" t="n"/>
       <c r="N20" s="11" t="n"/>
+      <c r="O20" s="11">
+        <f>IF(D20="","",IF(COUNTIFS($A$5:$A$404,A20,$D$5:$D$404,D20,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A20,$D$5:$D$404,D20,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n"/>
@@ -1145,6 +1215,10 @@
       <c r="L21" s="9" t="n"/>
       <c r="M21" s="9" t="n"/>
       <c r="N21" s="11" t="n"/>
+      <c r="O21" s="11">
+        <f>IF(D21="","",IF(COUNTIFS($A$5:$A$404,A21,$D$5:$D$404,D21,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A21,$D$5:$D$404,D21,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="n"/>
@@ -1164,6 +1238,10 @@
       <c r="L22" s="9" t="n"/>
       <c r="M22" s="9" t="n"/>
       <c r="N22" s="11" t="n"/>
+      <c r="O22" s="11">
+        <f>IF(D22="","",IF(COUNTIFS($A$5:$A$404,A22,$D$5:$D$404,D22,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A22,$D$5:$D$404,D22,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n"/>
@@ -1183,6 +1261,10 @@
       <c r="L23" s="9" t="n"/>
       <c r="M23" s="9" t="n"/>
       <c r="N23" s="11" t="n"/>
+      <c r="O23" s="11">
+        <f>IF(D23="","",IF(COUNTIFS($A$5:$A$404,A23,$D$5:$D$404,D23,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A23,$D$5:$D$404,D23,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="n"/>
@@ -1202,6 +1284,10 @@
       <c r="L24" s="9" t="n"/>
       <c r="M24" s="9" t="n"/>
       <c r="N24" s="11" t="n"/>
+      <c r="O24" s="11">
+        <f>IF(D24="","",IF(COUNTIFS($A$5:$A$404,A24,$D$5:$D$404,D24,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A24,$D$5:$D$404,D24,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="n"/>
@@ -1221,6 +1307,10 @@
       <c r="L25" s="9" t="n"/>
       <c r="M25" s="9" t="n"/>
       <c r="N25" s="11" t="n"/>
+      <c r="O25" s="11">
+        <f>IF(D25="","",IF(COUNTIFS($A$5:$A$404,A25,$D$5:$D$404,D25,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A25,$D$5:$D$404,D25,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n"/>
@@ -1240,6 +1330,10 @@
       <c r="L26" s="9" t="n"/>
       <c r="M26" s="9" t="n"/>
       <c r="N26" s="11" t="n"/>
+      <c r="O26" s="11">
+        <f>IF(D26="","",IF(COUNTIFS($A$5:$A$404,A26,$D$5:$D$404,D26,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A26,$D$5:$D$404,D26,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n"/>
@@ -1259,6 +1353,10 @@
       <c r="L27" s="9" t="n"/>
       <c r="M27" s="9" t="n"/>
       <c r="N27" s="11" t="n"/>
+      <c r="O27" s="11">
+        <f>IF(D27="","",IF(COUNTIFS($A$5:$A$404,A27,$D$5:$D$404,D27,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A27,$D$5:$D$404,D27,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n"/>
@@ -1278,6 +1376,10 @@
       <c r="L28" s="9" t="n"/>
       <c r="M28" s="9" t="n"/>
       <c r="N28" s="11" t="n"/>
+      <c r="O28" s="11">
+        <f>IF(D28="","",IF(COUNTIFS($A$5:$A$404,A28,$D$5:$D$404,D28,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A28,$D$5:$D$404,D28,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="n"/>
@@ -1297,6 +1399,10 @@
       <c r="L29" s="9" t="n"/>
       <c r="M29" s="9" t="n"/>
       <c r="N29" s="11" t="n"/>
+      <c r="O29" s="11">
+        <f>IF(D29="","",IF(COUNTIFS($A$5:$A$404,A29,$D$5:$D$404,D29,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A29,$D$5:$D$404,D29,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="n"/>
@@ -1316,6 +1422,10 @@
       <c r="L30" s="9" t="n"/>
       <c r="M30" s="9" t="n"/>
       <c r="N30" s="11" t="n"/>
+      <c r="O30" s="11">
+        <f>IF(D30="","",IF(COUNTIFS($A$5:$A$404,A30,$D$5:$D$404,D30,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A30,$D$5:$D$404,D30,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n"/>
@@ -1335,6 +1445,10 @@
       <c r="L31" s="9" t="n"/>
       <c r="M31" s="9" t="n"/>
       <c r="N31" s="11" t="n"/>
+      <c r="O31" s="11">
+        <f>IF(D31="","",IF(COUNTIFS($A$5:$A$404,A31,$D$5:$D$404,D31,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A31,$D$5:$D$404,D31,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n"/>
@@ -1354,6 +1468,10 @@
       <c r="L32" s="9" t="n"/>
       <c r="M32" s="9" t="n"/>
       <c r="N32" s="11" t="n"/>
+      <c r="O32" s="11">
+        <f>IF(D32="","",IF(COUNTIFS($A$5:$A$404,A32,$D$5:$D$404,D32,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A32,$D$5:$D$404,D32,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="n"/>
@@ -1373,6 +1491,10 @@
       <c r="L33" s="9" t="n"/>
       <c r="M33" s="9" t="n"/>
       <c r="N33" s="11" t="n"/>
+      <c r="O33" s="11">
+        <f>IF(D33="","",IF(COUNTIFS($A$5:$A$404,A33,$D$5:$D$404,D33,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A33,$D$5:$D$404,D33,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="n"/>
@@ -1392,6 +1514,10 @@
       <c r="L34" s="9" t="n"/>
       <c r="M34" s="9" t="n"/>
       <c r="N34" s="11" t="n"/>
+      <c r="O34" s="11">
+        <f>IF(D34="","",IF(COUNTIFS($A$5:$A$404,A34,$D$5:$D$404,D34,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A34,$D$5:$D$404,D34,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="n"/>
@@ -1411,6 +1537,10 @@
       <c r="L35" s="9" t="n"/>
       <c r="M35" s="9" t="n"/>
       <c r="N35" s="11" t="n"/>
+      <c r="O35" s="11">
+        <f>IF(D35="","",IF(COUNTIFS($A$5:$A$404,A35,$D$5:$D$404,D35,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A35,$D$5:$D$404,D35,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n"/>
@@ -1430,6 +1560,10 @@
       <c r="L36" s="9" t="n"/>
       <c r="M36" s="9" t="n"/>
       <c r="N36" s="11" t="n"/>
+      <c r="O36" s="11">
+        <f>IF(D36="","",IF(COUNTIFS($A$5:$A$404,A36,$D$5:$D$404,D36,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A36,$D$5:$D$404,D36,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n"/>
@@ -1449,6 +1583,10 @@
       <c r="L37" s="9" t="n"/>
       <c r="M37" s="9" t="n"/>
       <c r="N37" s="11" t="n"/>
+      <c r="O37" s="11">
+        <f>IF(D37="","",IF(COUNTIFS($A$5:$A$404,A37,$D$5:$D$404,D37,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A37,$D$5:$D$404,D37,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n"/>
@@ -1468,6 +1606,10 @@
       <c r="L38" s="9" t="n"/>
       <c r="M38" s="9" t="n"/>
       <c r="N38" s="11" t="n"/>
+      <c r="O38" s="11">
+        <f>IF(D38="","",IF(COUNTIFS($A$5:$A$404,A38,$D$5:$D$404,D38,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A38,$D$5:$D$404,D38,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="n"/>
@@ -1487,6 +1629,10 @@
       <c r="L39" s="9" t="n"/>
       <c r="M39" s="9" t="n"/>
       <c r="N39" s="11" t="n"/>
+      <c r="O39" s="11">
+        <f>IF(D39="","",IF(COUNTIFS($A$5:$A$404,A39,$D$5:$D$404,D39,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A39,$D$5:$D$404,D39,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="11" t="n"/>
@@ -1506,6 +1652,10 @@
       <c r="L40" s="9" t="n"/>
       <c r="M40" s="9" t="n"/>
       <c r="N40" s="11" t="n"/>
+      <c r="O40" s="11">
+        <f>IF(D40="","",IF(COUNTIFS($A$5:$A$404,A40,$D$5:$D$404,D40,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A40,$D$5:$D$404,D40,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="11" t="n"/>
@@ -1525,6 +1675,10 @@
       <c r="L41" s="9" t="n"/>
       <c r="M41" s="9" t="n"/>
       <c r="N41" s="11" t="n"/>
+      <c r="O41" s="11">
+        <f>IF(D41="","",IF(COUNTIFS($A$5:$A$404,A41,$D$5:$D$404,D41,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A41,$D$5:$D$404,D41,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="n"/>
@@ -1544,6 +1698,10 @@
       <c r="L42" s="9" t="n"/>
       <c r="M42" s="9" t="n"/>
       <c r="N42" s="11" t="n"/>
+      <c r="O42" s="11">
+        <f>IF(D42="","",IF(COUNTIFS($A$5:$A$404,A42,$D$5:$D$404,D42,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A42,$D$5:$D$404,D42,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="n"/>
@@ -1563,6 +1721,10 @@
       <c r="L43" s="9" t="n"/>
       <c r="M43" s="9" t="n"/>
       <c r="N43" s="11" t="n"/>
+      <c r="O43" s="11">
+        <f>IF(D43="","",IF(COUNTIFS($A$5:$A$404,A43,$D$5:$D$404,D43,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A43,$D$5:$D$404,D43,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="11" t="n"/>
@@ -1582,6 +1744,10 @@
       <c r="L44" s="9" t="n"/>
       <c r="M44" s="9" t="n"/>
       <c r="N44" s="11" t="n"/>
+      <c r="O44" s="11">
+        <f>IF(D44="","",IF(COUNTIFS($A$5:$A$404,A44,$D$5:$D$404,D44,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A44,$D$5:$D$404,D44,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="n"/>
@@ -1601,6 +1767,10 @@
       <c r="L45" s="9" t="n"/>
       <c r="M45" s="9" t="n"/>
       <c r="N45" s="11" t="n"/>
+      <c r="O45" s="11">
+        <f>IF(D45="","",IF(COUNTIFS($A$5:$A$404,A45,$D$5:$D$404,D45,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A45,$D$5:$D$404,D45,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="11" t="n"/>
@@ -1620,6 +1790,10 @@
       <c r="L46" s="9" t="n"/>
       <c r="M46" s="9" t="n"/>
       <c r="N46" s="11" t="n"/>
+      <c r="O46" s="11">
+        <f>IF(D46="","",IF(COUNTIFS($A$5:$A$404,A46,$D$5:$D$404,D46,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A46,$D$5:$D$404,D46,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="11" t="n"/>
@@ -1639,6 +1813,10 @@
       <c r="L47" s="9" t="n"/>
       <c r="M47" s="9" t="n"/>
       <c r="N47" s="11" t="n"/>
+      <c r="O47" s="11">
+        <f>IF(D47="","",IF(COUNTIFS($A$5:$A$404,A47,$D$5:$D$404,D47,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A47,$D$5:$D$404,D47,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="11" t="n"/>
@@ -1658,6 +1836,10 @@
       <c r="L48" s="9" t="n"/>
       <c r="M48" s="9" t="n"/>
       <c r="N48" s="11" t="n"/>
+      <c r="O48" s="11">
+        <f>IF(D48="","",IF(COUNTIFS($A$5:$A$404,A48,$D$5:$D$404,D48,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A48,$D$5:$D$404,D48,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="n"/>
@@ -1677,6 +1859,10 @@
       <c r="L49" s="9" t="n"/>
       <c r="M49" s="9" t="n"/>
       <c r="N49" s="11" t="n"/>
+      <c r="O49" s="11">
+        <f>IF(D49="","",IF(COUNTIFS($A$5:$A$404,A49,$D$5:$D$404,D49,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A49,$D$5:$D$404,D49,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="11" t="n"/>
@@ -1696,6 +1882,10 @@
       <c r="L50" s="9" t="n"/>
       <c r="M50" s="9" t="n"/>
       <c r="N50" s="11" t="n"/>
+      <c r="O50" s="11">
+        <f>IF(D50="","",IF(COUNTIFS($A$5:$A$404,A50,$D$5:$D$404,D50,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A50,$D$5:$D$404,D50,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="11" t="n"/>
@@ -1715,6 +1905,10 @@
       <c r="L51" s="9" t="n"/>
       <c r="M51" s="9" t="n"/>
       <c r="N51" s="11" t="n"/>
+      <c r="O51" s="11">
+        <f>IF(D51="","",IF(COUNTIFS($A$5:$A$404,A51,$D$5:$D$404,D51,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A51,$D$5:$D$404,D51,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n"/>
@@ -1734,6 +1928,10 @@
       <c r="L52" s="9" t="n"/>
       <c r="M52" s="9" t="n"/>
       <c r="N52" s="11" t="n"/>
+      <c r="O52" s="11">
+        <f>IF(D52="","",IF(COUNTIFS($A$5:$A$404,A52,$D$5:$D$404,D52,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A52,$D$5:$D$404,D52,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n"/>
@@ -1753,6 +1951,10 @@
       <c r="L53" s="9" t="n"/>
       <c r="M53" s="9" t="n"/>
       <c r="N53" s="11" t="n"/>
+      <c r="O53" s="11">
+        <f>IF(D53="","",IF(COUNTIFS($A$5:$A$404,A53,$D$5:$D$404,D53,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A53,$D$5:$D$404,D53,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n"/>
@@ -1772,6 +1974,10 @@
       <c r="L54" s="9" t="n"/>
       <c r="M54" s="9" t="n"/>
       <c r="N54" s="11" t="n"/>
+      <c r="O54" s="11">
+        <f>IF(D54="","",IF(COUNTIFS($A$5:$A$404,A54,$D$5:$D$404,D54,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A54,$D$5:$D$404,D54,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n"/>
@@ -1791,6 +1997,10 @@
       <c r="L55" s="9" t="n"/>
       <c r="M55" s="9" t="n"/>
       <c r="N55" s="11" t="n"/>
+      <c r="O55" s="11">
+        <f>IF(D55="","",IF(COUNTIFS($A$5:$A$404,A55,$D$5:$D$404,D55,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A55,$D$5:$D$404,D55,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n"/>
@@ -1810,6 +2020,10 @@
       <c r="L56" s="9" t="n"/>
       <c r="M56" s="9" t="n"/>
       <c r="N56" s="11" t="n"/>
+      <c r="O56" s="11">
+        <f>IF(D56="","",IF(COUNTIFS($A$5:$A$404,A56,$D$5:$D$404,D56,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A56,$D$5:$D$404,D56,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n"/>
@@ -1829,6 +2043,10 @@
       <c r="L57" s="9" t="n"/>
       <c r="M57" s="9" t="n"/>
       <c r="N57" s="11" t="n"/>
+      <c r="O57" s="11">
+        <f>IF(D57="","",IF(COUNTIFS($A$5:$A$404,A57,$D$5:$D$404,D57,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A57,$D$5:$D$404,D57,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n"/>
@@ -1848,6 +2066,10 @@
       <c r="L58" s="9" t="n"/>
       <c r="M58" s="9" t="n"/>
       <c r="N58" s="11" t="n"/>
+      <c r="O58" s="11">
+        <f>IF(D58="","",IF(COUNTIFS($A$5:$A$404,A58,$D$5:$D$404,D58,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A58,$D$5:$D$404,D58,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n"/>
@@ -1867,6 +2089,10 @@
       <c r="L59" s="9" t="n"/>
       <c r="M59" s="9" t="n"/>
       <c r="N59" s="11" t="n"/>
+      <c r="O59" s="11">
+        <f>IF(D59="","",IF(COUNTIFS($A$5:$A$404,A59,$D$5:$D$404,D59,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A59,$D$5:$D$404,D59,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n"/>
@@ -1886,6 +2112,10 @@
       <c r="L60" s="9" t="n"/>
       <c r="M60" s="9" t="n"/>
       <c r="N60" s="11" t="n"/>
+      <c r="O60" s="11">
+        <f>IF(D60="","",IF(COUNTIFS($A$5:$A$404,A60,$D$5:$D$404,D60,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A60,$D$5:$D$404,D60,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n"/>
@@ -1905,6 +2135,10 @@
       <c r="L61" s="9" t="n"/>
       <c r="M61" s="9" t="n"/>
       <c r="N61" s="11" t="n"/>
+      <c r="O61" s="11">
+        <f>IF(D61="","",IF(COUNTIFS($A$5:$A$404,A61,$D$5:$D$404,D61,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A61,$D$5:$D$404,D61,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n"/>
@@ -1924,6 +2158,10 @@
       <c r="L62" s="9" t="n"/>
       <c r="M62" s="9" t="n"/>
       <c r="N62" s="11" t="n"/>
+      <c r="O62" s="11">
+        <f>IF(D62="","",IF(COUNTIFS($A$5:$A$404,A62,$D$5:$D$404,D62,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A62,$D$5:$D$404,D62,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n"/>
@@ -1943,6 +2181,10 @@
       <c r="L63" s="9" t="n"/>
       <c r="M63" s="9" t="n"/>
       <c r="N63" s="11" t="n"/>
+      <c r="O63" s="11">
+        <f>IF(D63="","",IF(COUNTIFS($A$5:$A$404,A63,$D$5:$D$404,D63,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A63,$D$5:$D$404,D63,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n"/>
@@ -1962,6 +2204,10 @@
       <c r="L64" s="9" t="n"/>
       <c r="M64" s="9" t="n"/>
       <c r="N64" s="11" t="n"/>
+      <c r="O64" s="11">
+        <f>IF(D64="","",IF(COUNTIFS($A$5:$A$404,A64,$D$5:$D$404,D64,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A64,$D$5:$D$404,D64,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n"/>
@@ -1981,6 +2227,10 @@
       <c r="L65" s="9" t="n"/>
       <c r="M65" s="9" t="n"/>
       <c r="N65" s="11" t="n"/>
+      <c r="O65" s="11">
+        <f>IF(D65="","",IF(COUNTIFS($A$5:$A$404,A65,$D$5:$D$404,D65,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A65,$D$5:$D$404,D65,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="11" t="n"/>
@@ -2000,6 +2250,10 @@
       <c r="L66" s="9" t="n"/>
       <c r="M66" s="9" t="n"/>
       <c r="N66" s="11" t="n"/>
+      <c r="O66" s="11">
+        <f>IF(D66="","",IF(COUNTIFS($A$5:$A$404,A66,$D$5:$D$404,D66,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A66,$D$5:$D$404,D66,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="11" t="n"/>
@@ -2019,6 +2273,10 @@
       <c r="L67" s="9" t="n"/>
       <c r="M67" s="9" t="n"/>
       <c r="N67" s="11" t="n"/>
+      <c r="O67" s="11">
+        <f>IF(D67="","",IF(COUNTIFS($A$5:$A$404,A67,$D$5:$D$404,D67,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A67,$D$5:$D$404,D67,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="11" t="n"/>
@@ -2038,6 +2296,10 @@
       <c r="L68" s="9" t="n"/>
       <c r="M68" s="9" t="n"/>
       <c r="N68" s="11" t="n"/>
+      <c r="O68" s="11">
+        <f>IF(D68="","",IF(COUNTIFS($A$5:$A$404,A68,$D$5:$D$404,D68,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A68,$D$5:$D$404,D68,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="11" t="n"/>
@@ -2057,6 +2319,10 @@
       <c r="L69" s="9" t="n"/>
       <c r="M69" s="9" t="n"/>
       <c r="N69" s="11" t="n"/>
+      <c r="O69" s="11">
+        <f>IF(D69="","",IF(COUNTIFS($A$5:$A$404,A69,$D$5:$D$404,D69,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A69,$D$5:$D$404,D69,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="11" t="n"/>
@@ -2076,6 +2342,10 @@
       <c r="L70" s="9" t="n"/>
       <c r="M70" s="9" t="n"/>
       <c r="N70" s="11" t="n"/>
+      <c r="O70" s="11">
+        <f>IF(D70="","",IF(COUNTIFS($A$5:$A$404,A70,$D$5:$D$404,D70,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A70,$D$5:$D$404,D70,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="11" t="n"/>
@@ -2095,6 +2365,10 @@
       <c r="L71" s="9" t="n"/>
       <c r="M71" s="9" t="n"/>
       <c r="N71" s="11" t="n"/>
+      <c r="O71" s="11">
+        <f>IF(D71="","",IF(COUNTIFS($A$5:$A$404,A71,$D$5:$D$404,D71,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A71,$D$5:$D$404,D71,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="11" t="n"/>
@@ -2114,6 +2388,10 @@
       <c r="L72" s="9" t="n"/>
       <c r="M72" s="9" t="n"/>
       <c r="N72" s="11" t="n"/>
+      <c r="O72" s="11">
+        <f>IF(D72="","",IF(COUNTIFS($A$5:$A$404,A72,$D$5:$D$404,D72,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A72,$D$5:$D$404,D72,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="11" t="n"/>
@@ -2133,6 +2411,10 @@
       <c r="L73" s="9" t="n"/>
       <c r="M73" s="9" t="n"/>
       <c r="N73" s="11" t="n"/>
+      <c r="O73" s="11">
+        <f>IF(D73="","",IF(COUNTIFS($A$5:$A$404,A73,$D$5:$D$404,D73,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A73,$D$5:$D$404,D73,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="11" t="n"/>
@@ -2152,6 +2434,10 @@
       <c r="L74" s="9" t="n"/>
       <c r="M74" s="9" t="n"/>
       <c r="N74" s="11" t="n"/>
+      <c r="O74" s="11">
+        <f>IF(D74="","",IF(COUNTIFS($A$5:$A$404,A74,$D$5:$D$404,D74,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A74,$D$5:$D$404,D74,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="11" t="n"/>
@@ -2171,6 +2457,10 @@
       <c r="L75" s="9" t="n"/>
       <c r="M75" s="9" t="n"/>
       <c r="N75" s="11" t="n"/>
+      <c r="O75" s="11">
+        <f>IF(D75="","",IF(COUNTIFS($A$5:$A$404,A75,$D$5:$D$404,D75,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A75,$D$5:$D$404,D75,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="11" t="n"/>
@@ -2190,6 +2480,10 @@
       <c r="L76" s="9" t="n"/>
       <c r="M76" s="9" t="n"/>
       <c r="N76" s="11" t="n"/>
+      <c r="O76" s="11">
+        <f>IF(D76="","",IF(COUNTIFS($A$5:$A$404,A76,$D$5:$D$404,D76,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A76,$D$5:$D$404,D76,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="11" t="n"/>
@@ -2209,6 +2503,10 @@
       <c r="L77" s="9" t="n"/>
       <c r="M77" s="9" t="n"/>
       <c r="N77" s="11" t="n"/>
+      <c r="O77" s="11">
+        <f>IF(D77="","",IF(COUNTIFS($A$5:$A$404,A77,$D$5:$D$404,D77,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A77,$D$5:$D$404,D77,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="11" t="n"/>
@@ -2228,6 +2526,10 @@
       <c r="L78" s="9" t="n"/>
       <c r="M78" s="9" t="n"/>
       <c r="N78" s="11" t="n"/>
+      <c r="O78" s="11">
+        <f>IF(D78="","",IF(COUNTIFS($A$5:$A$404,A78,$D$5:$D$404,D78,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A78,$D$5:$D$404,D78,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="11" t="n"/>
@@ -2247,6 +2549,10 @@
       <c r="L79" s="9" t="n"/>
       <c r="M79" s="9" t="n"/>
       <c r="N79" s="11" t="n"/>
+      <c r="O79" s="11">
+        <f>IF(D79="","",IF(COUNTIFS($A$5:$A$404,A79,$D$5:$D$404,D79,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A79,$D$5:$D$404,D79,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="11" t="n"/>
@@ -2266,6 +2572,10 @@
       <c r="L80" s="9" t="n"/>
       <c r="M80" s="9" t="n"/>
       <c r="N80" s="11" t="n"/>
+      <c r="O80" s="11">
+        <f>IF(D80="","",IF(COUNTIFS($A$5:$A$404,A80,$D$5:$D$404,D80,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A80,$D$5:$D$404,D80,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="11" t="n"/>
@@ -2285,6 +2595,10 @@
       <c r="L81" s="9" t="n"/>
       <c r="M81" s="9" t="n"/>
       <c r="N81" s="11" t="n"/>
+      <c r="O81" s="11">
+        <f>IF(D81="","",IF(COUNTIFS($A$5:$A$404,A81,$D$5:$D$404,D81,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A81,$D$5:$D$404,D81,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="11" t="n"/>
@@ -2304,6 +2618,10 @@
       <c r="L82" s="9" t="n"/>
       <c r="M82" s="9" t="n"/>
       <c r="N82" s="11" t="n"/>
+      <c r="O82" s="11">
+        <f>IF(D82="","",IF(COUNTIFS($A$5:$A$404,A82,$D$5:$D$404,D82,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A82,$D$5:$D$404,D82,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="11" t="n"/>
@@ -2323,6 +2641,10 @@
       <c r="L83" s="9" t="n"/>
       <c r="M83" s="9" t="n"/>
       <c r="N83" s="11" t="n"/>
+      <c r="O83" s="11">
+        <f>IF(D83="","",IF(COUNTIFS($A$5:$A$404,A83,$D$5:$D$404,D83,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A83,$D$5:$D$404,D83,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="11" t="n"/>
@@ -2342,6 +2664,10 @@
       <c r="L84" s="9" t="n"/>
       <c r="M84" s="9" t="n"/>
       <c r="N84" s="11" t="n"/>
+      <c r="O84" s="11">
+        <f>IF(D84="","",IF(COUNTIFS($A$5:$A$404,A84,$D$5:$D$404,D84,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A84,$D$5:$D$404,D84,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="11" t="n"/>
@@ -2361,6 +2687,10 @@
       <c r="L85" s="9" t="n"/>
       <c r="M85" s="9" t="n"/>
       <c r="N85" s="11" t="n"/>
+      <c r="O85" s="11">
+        <f>IF(D85="","",IF(COUNTIFS($A$5:$A$404,A85,$D$5:$D$404,D85,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A85,$D$5:$D$404,D85,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="11" t="n"/>
@@ -2380,6 +2710,10 @@
       <c r="L86" s="9" t="n"/>
       <c r="M86" s="9" t="n"/>
       <c r="N86" s="11" t="n"/>
+      <c r="O86" s="11">
+        <f>IF(D86="","",IF(COUNTIFS($A$5:$A$404,A86,$D$5:$D$404,D86,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A86,$D$5:$D$404,D86,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="11" t="n"/>
@@ -2399,6 +2733,10 @@
       <c r="L87" s="9" t="n"/>
       <c r="M87" s="9" t="n"/>
       <c r="N87" s="11" t="n"/>
+      <c r="O87" s="11">
+        <f>IF(D87="","",IF(COUNTIFS($A$5:$A$404,A87,$D$5:$D$404,D87,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A87,$D$5:$D$404,D87,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="11" t="n"/>
@@ -2418,6 +2756,10 @@
       <c r="L88" s="9" t="n"/>
       <c r="M88" s="9" t="n"/>
       <c r="N88" s="11" t="n"/>
+      <c r="O88" s="11">
+        <f>IF(D88="","",IF(COUNTIFS($A$5:$A$404,A88,$D$5:$D$404,D88,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A88,$D$5:$D$404,D88,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="11" t="n"/>
@@ -2437,6 +2779,10 @@
       <c r="L89" s="9" t="n"/>
       <c r="M89" s="9" t="n"/>
       <c r="N89" s="11" t="n"/>
+      <c r="O89" s="11">
+        <f>IF(D89="","",IF(COUNTIFS($A$5:$A$404,A89,$D$5:$D$404,D89,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A89,$D$5:$D$404,D89,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="11" t="n"/>
@@ -2456,6 +2802,10 @@
       <c r="L90" s="9" t="n"/>
       <c r="M90" s="9" t="n"/>
       <c r="N90" s="11" t="n"/>
+      <c r="O90" s="11">
+        <f>IF(D90="","",IF(COUNTIFS($A$5:$A$404,A90,$D$5:$D$404,D90,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A90,$D$5:$D$404,D90,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="11" t="n"/>
@@ -2475,6 +2825,10 @@
       <c r="L91" s="9" t="n"/>
       <c r="M91" s="9" t="n"/>
       <c r="N91" s="11" t="n"/>
+      <c r="O91" s="11">
+        <f>IF(D91="","",IF(COUNTIFS($A$5:$A$404,A91,$D$5:$D$404,D91,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A91,$D$5:$D$404,D91,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="11" t="n"/>
@@ -2494,6 +2848,10 @@
       <c r="L92" s="9" t="n"/>
       <c r="M92" s="9" t="n"/>
       <c r="N92" s="11" t="n"/>
+      <c r="O92" s="11">
+        <f>IF(D92="","",IF(COUNTIFS($A$5:$A$404,A92,$D$5:$D$404,D92,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A92,$D$5:$D$404,D92,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="11" t="n"/>
@@ -2513,6 +2871,10 @@
       <c r="L93" s="9" t="n"/>
       <c r="M93" s="9" t="n"/>
       <c r="N93" s="11" t="n"/>
+      <c r="O93" s="11">
+        <f>IF(D93="","",IF(COUNTIFS($A$5:$A$404,A93,$D$5:$D$404,D93,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A93,$D$5:$D$404,D93,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="11" t="n"/>
@@ -2532,6 +2894,10 @@
       <c r="L94" s="9" t="n"/>
       <c r="M94" s="9" t="n"/>
       <c r="N94" s="11" t="n"/>
+      <c r="O94" s="11">
+        <f>IF(D94="","",IF(COUNTIFS($A$5:$A$404,A94,$D$5:$D$404,D94,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A94,$D$5:$D$404,D94,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="11" t="n"/>
@@ -2551,6 +2917,10 @@
       <c r="L95" s="9" t="n"/>
       <c r="M95" s="9" t="n"/>
       <c r="N95" s="11" t="n"/>
+      <c r="O95" s="11">
+        <f>IF(D95="","",IF(COUNTIFS($A$5:$A$404,A95,$D$5:$D$404,D95,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A95,$D$5:$D$404,D95,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="11" t="n"/>
@@ -2570,6 +2940,10 @@
       <c r="L96" s="9" t="n"/>
       <c r="M96" s="9" t="n"/>
       <c r="N96" s="11" t="n"/>
+      <c r="O96" s="11">
+        <f>IF(D96="","",IF(COUNTIFS($A$5:$A$404,A96,$D$5:$D$404,D96,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A96,$D$5:$D$404,D96,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="11" t="n"/>
@@ -2589,6 +2963,10 @@
       <c r="L97" s="9" t="n"/>
       <c r="M97" s="9" t="n"/>
       <c r="N97" s="11" t="n"/>
+      <c r="O97" s="11">
+        <f>IF(D97="","",IF(COUNTIFS($A$5:$A$404,A97,$D$5:$D$404,D97,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A97,$D$5:$D$404,D97,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="11" t="n"/>
@@ -2608,6 +2986,10 @@
       <c r="L98" s="9" t="n"/>
       <c r="M98" s="9" t="n"/>
       <c r="N98" s="11" t="n"/>
+      <c r="O98" s="11">
+        <f>IF(D98="","",IF(COUNTIFS($A$5:$A$404,A98,$D$5:$D$404,D98,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A98,$D$5:$D$404,D98,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="11" t="n"/>
@@ -2627,6 +3009,10 @@
       <c r="L99" s="9" t="n"/>
       <c r="M99" s="9" t="n"/>
       <c r="N99" s="11" t="n"/>
+      <c r="O99" s="11">
+        <f>IF(D99="","",IF(COUNTIFS($A$5:$A$404,A99,$D$5:$D$404,D99,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A99,$D$5:$D$404,D99,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="11" t="n"/>
@@ -2646,6 +3032,10 @@
       <c r="L100" s="9" t="n"/>
       <c r="M100" s="9" t="n"/>
       <c r="N100" s="11" t="n"/>
+      <c r="O100" s="11">
+        <f>IF(D100="","",IF(COUNTIFS($A$5:$A$404,A100,$D$5:$D$404,D100,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A100,$D$5:$D$404,D100,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="11" t="n"/>
@@ -2665,6 +3055,10 @@
       <c r="L101" s="9" t="n"/>
       <c r="M101" s="9" t="n"/>
       <c r="N101" s="11" t="n"/>
+      <c r="O101" s="11">
+        <f>IF(D101="","",IF(COUNTIFS($A$5:$A$404,A101,$D$5:$D$404,D101,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A101,$D$5:$D$404,D101,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="11" t="n"/>
@@ -2684,6 +3078,10 @@
       <c r="L102" s="9" t="n"/>
       <c r="M102" s="9" t="n"/>
       <c r="N102" s="11" t="n"/>
+      <c r="O102" s="11">
+        <f>IF(D102="","",IF(COUNTIFS($A$5:$A$404,A102,$D$5:$D$404,D102,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A102,$D$5:$D$404,D102,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="11" t="n"/>
@@ -2703,6 +3101,10 @@
       <c r="L103" s="9" t="n"/>
       <c r="M103" s="9" t="n"/>
       <c r="N103" s="11" t="n"/>
+      <c r="O103" s="11">
+        <f>IF(D103="","",IF(COUNTIFS($A$5:$A$404,A103,$D$5:$D$404,D103,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A103,$D$5:$D$404,D103,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="11" t="n"/>
@@ -2722,6 +3124,10 @@
       <c r="L104" s="9" t="n"/>
       <c r="M104" s="9" t="n"/>
       <c r="N104" s="11" t="n"/>
+      <c r="O104" s="11">
+        <f>IF(D104="","",IF(COUNTIFS($A$5:$A$404,A104,$D$5:$D$404,D104,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A104,$D$5:$D$404,D104,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="11" t="n"/>
@@ -2741,6 +3147,10 @@
       <c r="L105" s="9" t="n"/>
       <c r="M105" s="9" t="n"/>
       <c r="N105" s="11" t="n"/>
+      <c r="O105" s="11">
+        <f>IF(D105="","",IF(COUNTIFS($A$5:$A$404,A105,$D$5:$D$404,D105,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A105,$D$5:$D$404,D105,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="11" t="n"/>
@@ -2760,6 +3170,10 @@
       <c r="L106" s="9" t="n"/>
       <c r="M106" s="9" t="n"/>
       <c r="N106" s="11" t="n"/>
+      <c r="O106" s="11">
+        <f>IF(D106="","",IF(COUNTIFS($A$5:$A$404,A106,$D$5:$D$404,D106,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A106,$D$5:$D$404,D106,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="11" t="n"/>
@@ -2779,6 +3193,10 @@
       <c r="L107" s="9" t="n"/>
       <c r="M107" s="9" t="n"/>
       <c r="N107" s="11" t="n"/>
+      <c r="O107" s="11">
+        <f>IF(D107="","",IF(COUNTIFS($A$5:$A$404,A107,$D$5:$D$404,D107,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A107,$D$5:$D$404,D107,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="11" t="n"/>
@@ -2798,6 +3216,10 @@
       <c r="L108" s="9" t="n"/>
       <c r="M108" s="9" t="n"/>
       <c r="N108" s="11" t="n"/>
+      <c r="O108" s="11">
+        <f>IF(D108="","",IF(COUNTIFS($A$5:$A$404,A108,$D$5:$D$404,D108,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A108,$D$5:$D$404,D108,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="11" t="n"/>
@@ -2817,6 +3239,10 @@
       <c r="L109" s="9" t="n"/>
       <c r="M109" s="9" t="n"/>
       <c r="N109" s="11" t="n"/>
+      <c r="O109" s="11">
+        <f>IF(D109="","",IF(COUNTIFS($A$5:$A$404,A109,$D$5:$D$404,D109,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A109,$D$5:$D$404,D109,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="11" t="n"/>
@@ -2836,6 +3262,10 @@
       <c r="L110" s="9" t="n"/>
       <c r="M110" s="9" t="n"/>
       <c r="N110" s="11" t="n"/>
+      <c r="O110" s="11">
+        <f>IF(D110="","",IF(COUNTIFS($A$5:$A$404,A110,$D$5:$D$404,D110,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A110,$D$5:$D$404,D110,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="11" t="n"/>
@@ -2855,6 +3285,10 @@
       <c r="L111" s="9" t="n"/>
       <c r="M111" s="9" t="n"/>
       <c r="N111" s="11" t="n"/>
+      <c r="O111" s="11">
+        <f>IF(D111="","",IF(COUNTIFS($A$5:$A$404,A111,$D$5:$D$404,D111,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A111,$D$5:$D$404,D111,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="11" t="n"/>
@@ -2874,6 +3308,10 @@
       <c r="L112" s="9" t="n"/>
       <c r="M112" s="9" t="n"/>
       <c r="N112" s="11" t="n"/>
+      <c r="O112" s="11">
+        <f>IF(D112="","",IF(COUNTIFS($A$5:$A$404,A112,$D$5:$D$404,D112,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A112,$D$5:$D$404,D112,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="11" t="n"/>
@@ -2893,6 +3331,10 @@
       <c r="L113" s="9" t="n"/>
       <c r="M113" s="9" t="n"/>
       <c r="N113" s="11" t="n"/>
+      <c r="O113" s="11">
+        <f>IF(D113="","",IF(COUNTIFS($A$5:$A$404,A113,$D$5:$D$404,D113,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A113,$D$5:$D$404,D113,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="11" t="n"/>
@@ -2912,6 +3354,10 @@
       <c r="L114" s="9" t="n"/>
       <c r="M114" s="9" t="n"/>
       <c r="N114" s="11" t="n"/>
+      <c r="O114" s="11">
+        <f>IF(D114="","",IF(COUNTIFS($A$5:$A$404,A114,$D$5:$D$404,D114,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A114,$D$5:$D$404,D114,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="11" t="n"/>
@@ -2931,6 +3377,10 @@
       <c r="L115" s="9" t="n"/>
       <c r="M115" s="9" t="n"/>
       <c r="N115" s="11" t="n"/>
+      <c r="O115" s="11">
+        <f>IF(D115="","",IF(COUNTIFS($A$5:$A$404,A115,$D$5:$D$404,D115,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A115,$D$5:$D$404,D115,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="11" t="n"/>
@@ -2950,6 +3400,10 @@
       <c r="L116" s="9" t="n"/>
       <c r="M116" s="9" t="n"/>
       <c r="N116" s="11" t="n"/>
+      <c r="O116" s="11">
+        <f>IF(D116="","",IF(COUNTIFS($A$5:$A$404,A116,$D$5:$D$404,D116,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A116,$D$5:$D$404,D116,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="11" t="n"/>
@@ -2969,6 +3423,10 @@
       <c r="L117" s="9" t="n"/>
       <c r="M117" s="9" t="n"/>
       <c r="N117" s="11" t="n"/>
+      <c r="O117" s="11">
+        <f>IF(D117="","",IF(COUNTIFS($A$5:$A$404,A117,$D$5:$D$404,D117,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A117,$D$5:$D$404,D117,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="11" t="n"/>
@@ -2988,6 +3446,10 @@
       <c r="L118" s="9" t="n"/>
       <c r="M118" s="9" t="n"/>
       <c r="N118" s="11" t="n"/>
+      <c r="O118" s="11">
+        <f>IF(D118="","",IF(COUNTIFS($A$5:$A$404,A118,$D$5:$D$404,D118,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A118,$D$5:$D$404,D118,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="11" t="n"/>
@@ -3007,6 +3469,10 @@
       <c r="L119" s="9" t="n"/>
       <c r="M119" s="9" t="n"/>
       <c r="N119" s="11" t="n"/>
+      <c r="O119" s="11">
+        <f>IF(D119="","",IF(COUNTIFS($A$5:$A$404,A119,$D$5:$D$404,D119,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A119,$D$5:$D$404,D119,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="11" t="n"/>
@@ -3026,6 +3492,10 @@
       <c r="L120" s="9" t="n"/>
       <c r="M120" s="9" t="n"/>
       <c r="N120" s="11" t="n"/>
+      <c r="O120" s="11">
+        <f>IF(D120="","",IF(COUNTIFS($A$5:$A$404,A120,$D$5:$D$404,D120,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A120,$D$5:$D$404,D120,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="11" t="n"/>
@@ -3045,6 +3515,10 @@
       <c r="L121" s="9" t="n"/>
       <c r="M121" s="9" t="n"/>
       <c r="N121" s="11" t="n"/>
+      <c r="O121" s="11">
+        <f>IF(D121="","",IF(COUNTIFS($A$5:$A$404,A121,$D$5:$D$404,D121,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A121,$D$5:$D$404,D121,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="11" t="n"/>
@@ -3064,6 +3538,10 @@
       <c r="L122" s="9" t="n"/>
       <c r="M122" s="9" t="n"/>
       <c r="N122" s="11" t="n"/>
+      <c r="O122" s="11">
+        <f>IF(D122="","",IF(COUNTIFS($A$5:$A$404,A122,$D$5:$D$404,D122,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A122,$D$5:$D$404,D122,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="11" t="n"/>
@@ -3083,6 +3561,10 @@
       <c r="L123" s="9" t="n"/>
       <c r="M123" s="9" t="n"/>
       <c r="N123" s="11" t="n"/>
+      <c r="O123" s="11">
+        <f>IF(D123="","",IF(COUNTIFS($A$5:$A$404,A123,$D$5:$D$404,D123,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A123,$D$5:$D$404,D123,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="11" t="n"/>
@@ -3102,6 +3584,10 @@
       <c r="L124" s="9" t="n"/>
       <c r="M124" s="9" t="n"/>
       <c r="N124" s="11" t="n"/>
+      <c r="O124" s="11">
+        <f>IF(D124="","",IF(COUNTIFS($A$5:$A$404,A124,$D$5:$D$404,D124,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A124,$D$5:$D$404,D124,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="11" t="n"/>
@@ -3121,6 +3607,10 @@
       <c r="L125" s="9" t="n"/>
       <c r="M125" s="9" t="n"/>
       <c r="N125" s="11" t="n"/>
+      <c r="O125" s="11">
+        <f>IF(D125="","",IF(COUNTIFS($A$5:$A$404,A125,$D$5:$D$404,D125,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A125,$D$5:$D$404,D125,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="11" t="n"/>
@@ -3140,6 +3630,10 @@
       <c r="L126" s="9" t="n"/>
       <c r="M126" s="9" t="n"/>
       <c r="N126" s="11" t="n"/>
+      <c r="O126" s="11">
+        <f>IF(D126="","",IF(COUNTIFS($A$5:$A$404,A126,$D$5:$D$404,D126,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A126,$D$5:$D$404,D126,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="11" t="n"/>
@@ -3159,6 +3653,10 @@
       <c r="L127" s="9" t="n"/>
       <c r="M127" s="9" t="n"/>
       <c r="N127" s="11" t="n"/>
+      <c r="O127" s="11">
+        <f>IF(D127="","",IF(COUNTIFS($A$5:$A$404,A127,$D$5:$D$404,D127,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A127,$D$5:$D$404,D127,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="11" t="n"/>
@@ -3178,6 +3676,10 @@
       <c r="L128" s="9" t="n"/>
       <c r="M128" s="9" t="n"/>
       <c r="N128" s="11" t="n"/>
+      <c r="O128" s="11">
+        <f>IF(D128="","",IF(COUNTIFS($A$5:$A$404,A128,$D$5:$D$404,D128,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A128,$D$5:$D$404,D128,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="11" t="n"/>
@@ -3197,6 +3699,10 @@
       <c r="L129" s="9" t="n"/>
       <c r="M129" s="9" t="n"/>
       <c r="N129" s="11" t="n"/>
+      <c r="O129" s="11">
+        <f>IF(D129="","",IF(COUNTIFS($A$5:$A$404,A129,$D$5:$D$404,D129,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A129,$D$5:$D$404,D129,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="11" t="n"/>
@@ -3216,6 +3722,10 @@
       <c r="L130" s="9" t="n"/>
       <c r="M130" s="9" t="n"/>
       <c r="N130" s="11" t="n"/>
+      <c r="O130" s="11">
+        <f>IF(D130="","",IF(COUNTIFS($A$5:$A$404,A130,$D$5:$D$404,D130,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A130,$D$5:$D$404,D130,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="11" t="n"/>
@@ -3235,6 +3745,10 @@
       <c r="L131" s="9" t="n"/>
       <c r="M131" s="9" t="n"/>
       <c r="N131" s="11" t="n"/>
+      <c r="O131" s="11">
+        <f>IF(D131="","",IF(COUNTIFS($A$5:$A$404,A131,$D$5:$D$404,D131,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A131,$D$5:$D$404,D131,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="11" t="n"/>
@@ -3254,6 +3768,10 @@
       <c r="L132" s="9" t="n"/>
       <c r="M132" s="9" t="n"/>
       <c r="N132" s="11" t="n"/>
+      <c r="O132" s="11">
+        <f>IF(D132="","",IF(COUNTIFS($A$5:$A$404,A132,$D$5:$D$404,D132,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A132,$D$5:$D$404,D132,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="11" t="n"/>
@@ -3273,6 +3791,10 @@
       <c r="L133" s="9" t="n"/>
       <c r="M133" s="9" t="n"/>
       <c r="N133" s="11" t="n"/>
+      <c r="O133" s="11">
+        <f>IF(D133="","",IF(COUNTIFS($A$5:$A$404,A133,$D$5:$D$404,D133,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A133,$D$5:$D$404,D133,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="11" t="n"/>
@@ -3292,6 +3814,10 @@
       <c r="L134" s="9" t="n"/>
       <c r="M134" s="9" t="n"/>
       <c r="N134" s="11" t="n"/>
+      <c r="O134" s="11">
+        <f>IF(D134="","",IF(COUNTIFS($A$5:$A$404,A134,$D$5:$D$404,D134,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A134,$D$5:$D$404,D134,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="11" t="n"/>
@@ -3311,6 +3837,10 @@
       <c r="L135" s="9" t="n"/>
       <c r="M135" s="9" t="n"/>
       <c r="N135" s="11" t="n"/>
+      <c r="O135" s="11">
+        <f>IF(D135="","",IF(COUNTIFS($A$5:$A$404,A135,$D$5:$D$404,D135,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A135,$D$5:$D$404,D135,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="11" t="n"/>
@@ -3330,6 +3860,10 @@
       <c r="L136" s="9" t="n"/>
       <c r="M136" s="9" t="n"/>
       <c r="N136" s="11" t="n"/>
+      <c r="O136" s="11">
+        <f>IF(D136="","",IF(COUNTIFS($A$5:$A$404,A136,$D$5:$D$404,D136,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A136,$D$5:$D$404,D136,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="11" t="n"/>
@@ -3349,6 +3883,10 @@
       <c r="L137" s="9" t="n"/>
       <c r="M137" s="9" t="n"/>
       <c r="N137" s="11" t="n"/>
+      <c r="O137" s="11">
+        <f>IF(D137="","",IF(COUNTIFS($A$5:$A$404,A137,$D$5:$D$404,D137,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A137,$D$5:$D$404,D137,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="11" t="n"/>
@@ -3368,6 +3906,10 @@
       <c r="L138" s="9" t="n"/>
       <c r="M138" s="9" t="n"/>
       <c r="N138" s="11" t="n"/>
+      <c r="O138" s="11">
+        <f>IF(D138="","",IF(COUNTIFS($A$5:$A$404,A138,$D$5:$D$404,D138,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A138,$D$5:$D$404,D138,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="11" t="n"/>
@@ -3387,6 +3929,10 @@
       <c r="L139" s="9" t="n"/>
       <c r="M139" s="9" t="n"/>
       <c r="N139" s="11" t="n"/>
+      <c r="O139" s="11">
+        <f>IF(D139="","",IF(COUNTIFS($A$5:$A$404,A139,$D$5:$D$404,D139,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A139,$D$5:$D$404,D139,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="11" t="n"/>
@@ -3406,6 +3952,10 @@
       <c r="L140" s="9" t="n"/>
       <c r="M140" s="9" t="n"/>
       <c r="N140" s="11" t="n"/>
+      <c r="O140" s="11">
+        <f>IF(D140="","",IF(COUNTIFS($A$5:$A$404,A140,$D$5:$D$404,D140,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A140,$D$5:$D$404,D140,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="11" t="n"/>
@@ -3425,6 +3975,10 @@
       <c r="L141" s="9" t="n"/>
       <c r="M141" s="9" t="n"/>
       <c r="N141" s="11" t="n"/>
+      <c r="O141" s="11">
+        <f>IF(D141="","",IF(COUNTIFS($A$5:$A$404,A141,$D$5:$D$404,D141,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A141,$D$5:$D$404,D141,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="11" t="n"/>
@@ -3444,6 +3998,10 @@
       <c r="L142" s="9" t="n"/>
       <c r="M142" s="9" t="n"/>
       <c r="N142" s="11" t="n"/>
+      <c r="O142" s="11">
+        <f>IF(D142="","",IF(COUNTIFS($A$5:$A$404,A142,$D$5:$D$404,D142,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A142,$D$5:$D$404,D142,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="11" t="n"/>
@@ -3463,6 +4021,10 @@
       <c r="L143" s="9" t="n"/>
       <c r="M143" s="9" t="n"/>
       <c r="N143" s="11" t="n"/>
+      <c r="O143" s="11">
+        <f>IF(D143="","",IF(COUNTIFS($A$5:$A$404,A143,$D$5:$D$404,D143,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A143,$D$5:$D$404,D143,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="11" t="n"/>
@@ -3482,6 +4044,10 @@
       <c r="L144" s="9" t="n"/>
       <c r="M144" s="9" t="n"/>
       <c r="N144" s="11" t="n"/>
+      <c r="O144" s="11">
+        <f>IF(D144="","",IF(COUNTIFS($A$5:$A$404,A144,$D$5:$D$404,D144,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A144,$D$5:$D$404,D144,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="11" t="n"/>
@@ -3501,6 +4067,10 @@
       <c r="L145" s="9" t="n"/>
       <c r="M145" s="9" t="n"/>
       <c r="N145" s="11" t="n"/>
+      <c r="O145" s="11">
+        <f>IF(D145="","",IF(COUNTIFS($A$5:$A$404,A145,$D$5:$D$404,D145,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A145,$D$5:$D$404,D145,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="11" t="n"/>
@@ -3520,6 +4090,10 @@
       <c r="L146" s="9" t="n"/>
       <c r="M146" s="9" t="n"/>
       <c r="N146" s="11" t="n"/>
+      <c r="O146" s="11">
+        <f>IF(D146="","",IF(COUNTIFS($A$5:$A$404,A146,$D$5:$D$404,D146,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A146,$D$5:$D$404,D146,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="11" t="n"/>
@@ -3539,6 +4113,10 @@
       <c r="L147" s="9" t="n"/>
       <c r="M147" s="9" t="n"/>
       <c r="N147" s="11" t="n"/>
+      <c r="O147" s="11">
+        <f>IF(D147="","",IF(COUNTIFS($A$5:$A$404,A147,$D$5:$D$404,D147,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A147,$D$5:$D$404,D147,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="11" t="n"/>
@@ -3558,6 +4136,10 @@
       <c r="L148" s="9" t="n"/>
       <c r="M148" s="9" t="n"/>
       <c r="N148" s="11" t="n"/>
+      <c r="O148" s="11">
+        <f>IF(D148="","",IF(COUNTIFS($A$5:$A$404,A148,$D$5:$D$404,D148,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A148,$D$5:$D$404,D148,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="11" t="n"/>
@@ -3577,6 +4159,10 @@
       <c r="L149" s="9" t="n"/>
       <c r="M149" s="9" t="n"/>
       <c r="N149" s="11" t="n"/>
+      <c r="O149" s="11">
+        <f>IF(D149="","",IF(COUNTIFS($A$5:$A$404,A149,$D$5:$D$404,D149,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A149,$D$5:$D$404,D149,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="11" t="n"/>
@@ -3596,6 +4182,10 @@
       <c r="L150" s="9" t="n"/>
       <c r="M150" s="9" t="n"/>
       <c r="N150" s="11" t="n"/>
+      <c r="O150" s="11">
+        <f>IF(D150="","",IF(COUNTIFS($A$5:$A$404,A150,$D$5:$D$404,D150,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A150,$D$5:$D$404,D150,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="11" t="n"/>
@@ -3615,6 +4205,10 @@
       <c r="L151" s="9" t="n"/>
       <c r="M151" s="9" t="n"/>
       <c r="N151" s="11" t="n"/>
+      <c r="O151" s="11">
+        <f>IF(D151="","",IF(COUNTIFS($A$5:$A$404,A151,$D$5:$D$404,D151,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A151,$D$5:$D$404,D151,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="11" t="n"/>
@@ -3634,6 +4228,10 @@
       <c r="L152" s="9" t="n"/>
       <c r="M152" s="9" t="n"/>
       <c r="N152" s="11" t="n"/>
+      <c r="O152" s="11">
+        <f>IF(D152="","",IF(COUNTIFS($A$5:$A$404,A152,$D$5:$D$404,D152,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A152,$D$5:$D$404,D152,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="11" t="n"/>
@@ -3653,6 +4251,10 @@
       <c r="L153" s="9" t="n"/>
       <c r="M153" s="9" t="n"/>
       <c r="N153" s="11" t="n"/>
+      <c r="O153" s="11">
+        <f>IF(D153="","",IF(COUNTIFS($A$5:$A$404,A153,$D$5:$D$404,D153,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A153,$D$5:$D$404,D153,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="11" t="n"/>
@@ -3672,6 +4274,10 @@
       <c r="L154" s="9" t="n"/>
       <c r="M154" s="9" t="n"/>
       <c r="N154" s="11" t="n"/>
+      <c r="O154" s="11">
+        <f>IF(D154="","",IF(COUNTIFS($A$5:$A$404,A154,$D$5:$D$404,D154,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A154,$D$5:$D$404,D154,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="11" t="n"/>
@@ -3691,6 +4297,10 @@
       <c r="L155" s="9" t="n"/>
       <c r="M155" s="9" t="n"/>
       <c r="N155" s="11" t="n"/>
+      <c r="O155" s="11">
+        <f>IF(D155="","",IF(COUNTIFS($A$5:$A$404,A155,$D$5:$D$404,D155,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A155,$D$5:$D$404,D155,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="11" t="n"/>
@@ -3710,6 +4320,10 @@
       <c r="L156" s="9" t="n"/>
       <c r="M156" s="9" t="n"/>
       <c r="N156" s="11" t="n"/>
+      <c r="O156" s="11">
+        <f>IF(D156="","",IF(COUNTIFS($A$5:$A$404,A156,$D$5:$D$404,D156,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A156,$D$5:$D$404,D156,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="11" t="n"/>
@@ -3729,6 +4343,10 @@
       <c r="L157" s="9" t="n"/>
       <c r="M157" s="9" t="n"/>
       <c r="N157" s="11" t="n"/>
+      <c r="O157" s="11">
+        <f>IF(D157="","",IF(COUNTIFS($A$5:$A$404,A157,$D$5:$D$404,D157,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A157,$D$5:$D$404,D157,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="11" t="n"/>
@@ -3748,6 +4366,10 @@
       <c r="L158" s="9" t="n"/>
       <c r="M158" s="9" t="n"/>
       <c r="N158" s="11" t="n"/>
+      <c r="O158" s="11">
+        <f>IF(D158="","",IF(COUNTIFS($A$5:$A$404,A158,$D$5:$D$404,D158,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A158,$D$5:$D$404,D158,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="11" t="n"/>
@@ -3767,6 +4389,10 @@
       <c r="L159" s="9" t="n"/>
       <c r="M159" s="9" t="n"/>
       <c r="N159" s="11" t="n"/>
+      <c r="O159" s="11">
+        <f>IF(D159="","",IF(COUNTIFS($A$5:$A$404,A159,$D$5:$D$404,D159,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A159,$D$5:$D$404,D159,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="11" t="n"/>
@@ -3786,6 +4412,10 @@
       <c r="L160" s="9" t="n"/>
       <c r="M160" s="9" t="n"/>
       <c r="N160" s="11" t="n"/>
+      <c r="O160" s="11">
+        <f>IF(D160="","",IF(COUNTIFS($A$5:$A$404,A160,$D$5:$D$404,D160,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A160,$D$5:$D$404,D160,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="11" t="n"/>
@@ -3805,6 +4435,10 @@
       <c r="L161" s="9" t="n"/>
       <c r="M161" s="9" t="n"/>
       <c r="N161" s="11" t="n"/>
+      <c r="O161" s="11">
+        <f>IF(D161="","",IF(COUNTIFS($A$5:$A$404,A161,$D$5:$D$404,D161,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A161,$D$5:$D$404,D161,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="11" t="n"/>
@@ -3824,6 +4458,10 @@
       <c r="L162" s="9" t="n"/>
       <c r="M162" s="9" t="n"/>
       <c r="N162" s="11" t="n"/>
+      <c r="O162" s="11">
+        <f>IF(D162="","",IF(COUNTIFS($A$5:$A$404,A162,$D$5:$D$404,D162,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A162,$D$5:$D$404,D162,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="11" t="n"/>
@@ -3843,6 +4481,10 @@
       <c r="L163" s="9" t="n"/>
       <c r="M163" s="9" t="n"/>
       <c r="N163" s="11" t="n"/>
+      <c r="O163" s="11">
+        <f>IF(D163="","",IF(COUNTIFS($A$5:$A$404,A163,$D$5:$D$404,D163,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A163,$D$5:$D$404,D163,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="11" t="n"/>
@@ -3862,6 +4504,10 @@
       <c r="L164" s="9" t="n"/>
       <c r="M164" s="9" t="n"/>
       <c r="N164" s="11" t="n"/>
+      <c r="O164" s="11">
+        <f>IF(D164="","",IF(COUNTIFS($A$5:$A$404,A164,$D$5:$D$404,D164,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A164,$D$5:$D$404,D164,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="11" t="n"/>
@@ -3881,6 +4527,10 @@
       <c r="L165" s="9" t="n"/>
       <c r="M165" s="9" t="n"/>
       <c r="N165" s="11" t="n"/>
+      <c r="O165" s="11">
+        <f>IF(D165="","",IF(COUNTIFS($A$5:$A$404,A165,$D$5:$D$404,D165,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A165,$D$5:$D$404,D165,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="11" t="n"/>
@@ -3900,6 +4550,10 @@
       <c r="L166" s="9" t="n"/>
       <c r="M166" s="9" t="n"/>
       <c r="N166" s="11" t="n"/>
+      <c r="O166" s="11">
+        <f>IF(D166="","",IF(COUNTIFS($A$5:$A$404,A166,$D$5:$D$404,D166,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A166,$D$5:$D$404,D166,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="11" t="n"/>
@@ -3919,6 +4573,10 @@
       <c r="L167" s="9" t="n"/>
       <c r="M167" s="9" t="n"/>
       <c r="N167" s="11" t="n"/>
+      <c r="O167" s="11">
+        <f>IF(D167="","",IF(COUNTIFS($A$5:$A$404,A167,$D$5:$D$404,D167,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A167,$D$5:$D$404,D167,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="11" t="n"/>
@@ -3938,6 +4596,10 @@
       <c r="L168" s="9" t="n"/>
       <c r="M168" s="9" t="n"/>
       <c r="N168" s="11" t="n"/>
+      <c r="O168" s="11">
+        <f>IF(D168="","",IF(COUNTIFS($A$5:$A$404,A168,$D$5:$D$404,D168,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A168,$D$5:$D$404,D168,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="11" t="n"/>
@@ -3957,6 +4619,10 @@
       <c r="L169" s="9" t="n"/>
       <c r="M169" s="9" t="n"/>
       <c r="N169" s="11" t="n"/>
+      <c r="O169" s="11">
+        <f>IF(D169="","",IF(COUNTIFS($A$5:$A$404,A169,$D$5:$D$404,D169,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A169,$D$5:$D$404,D169,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="11" t="n"/>
@@ -3976,6 +4642,10 @@
       <c r="L170" s="9" t="n"/>
       <c r="M170" s="9" t="n"/>
       <c r="N170" s="11" t="n"/>
+      <c r="O170" s="11">
+        <f>IF(D170="","",IF(COUNTIFS($A$5:$A$404,A170,$D$5:$D$404,D170,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A170,$D$5:$D$404,D170,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="11" t="n"/>
@@ -3995,6 +4665,10 @@
       <c r="L171" s="9" t="n"/>
       <c r="M171" s="9" t="n"/>
       <c r="N171" s="11" t="n"/>
+      <c r="O171" s="11">
+        <f>IF(D171="","",IF(COUNTIFS($A$5:$A$404,A171,$D$5:$D$404,D171,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A171,$D$5:$D$404,D171,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="11" t="n"/>
@@ -4014,6 +4688,10 @@
       <c r="L172" s="9" t="n"/>
       <c r="M172" s="9" t="n"/>
       <c r="N172" s="11" t="n"/>
+      <c r="O172" s="11">
+        <f>IF(D172="","",IF(COUNTIFS($A$5:$A$404,A172,$D$5:$D$404,D172,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A172,$D$5:$D$404,D172,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="11" t="n"/>
@@ -4033,6 +4711,10 @@
       <c r="L173" s="9" t="n"/>
       <c r="M173" s="9" t="n"/>
       <c r="N173" s="11" t="n"/>
+      <c r="O173" s="11">
+        <f>IF(D173="","",IF(COUNTIFS($A$5:$A$404,A173,$D$5:$D$404,D173,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A173,$D$5:$D$404,D173,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="11" t="n"/>
@@ -4052,6 +4734,10 @@
       <c r="L174" s="9" t="n"/>
       <c r="M174" s="9" t="n"/>
       <c r="N174" s="11" t="n"/>
+      <c r="O174" s="11">
+        <f>IF(D174="","",IF(COUNTIFS($A$5:$A$404,A174,$D$5:$D$404,D174,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A174,$D$5:$D$404,D174,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="11" t="n"/>
@@ -4071,6 +4757,10 @@
       <c r="L175" s="9" t="n"/>
       <c r="M175" s="9" t="n"/>
       <c r="N175" s="11" t="n"/>
+      <c r="O175" s="11">
+        <f>IF(D175="","",IF(COUNTIFS($A$5:$A$404,A175,$D$5:$D$404,D175,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A175,$D$5:$D$404,D175,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="11" t="n"/>
@@ -4090,6 +4780,10 @@
       <c r="L176" s="9" t="n"/>
       <c r="M176" s="9" t="n"/>
       <c r="N176" s="11" t="n"/>
+      <c r="O176" s="11">
+        <f>IF(D176="","",IF(COUNTIFS($A$5:$A$404,A176,$D$5:$D$404,D176,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A176,$D$5:$D$404,D176,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="11" t="n"/>
@@ -4109,6 +4803,10 @@
       <c r="L177" s="9" t="n"/>
       <c r="M177" s="9" t="n"/>
       <c r="N177" s="11" t="n"/>
+      <c r="O177" s="11">
+        <f>IF(D177="","",IF(COUNTIFS($A$5:$A$404,A177,$D$5:$D$404,D177,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A177,$D$5:$D$404,D177,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="11" t="n"/>
@@ -4128,6 +4826,10 @@
       <c r="L178" s="9" t="n"/>
       <c r="M178" s="9" t="n"/>
       <c r="N178" s="11" t="n"/>
+      <c r="O178" s="11">
+        <f>IF(D178="","",IF(COUNTIFS($A$5:$A$404,A178,$D$5:$D$404,D178,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A178,$D$5:$D$404,D178,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="11" t="n"/>
@@ -4147,6 +4849,10 @@
       <c r="L179" s="9" t="n"/>
       <c r="M179" s="9" t="n"/>
       <c r="N179" s="11" t="n"/>
+      <c r="O179" s="11">
+        <f>IF(D179="","",IF(COUNTIFS($A$5:$A$404,A179,$D$5:$D$404,D179,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A179,$D$5:$D$404,D179,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="11" t="n"/>
@@ -4166,6 +4872,10 @@
       <c r="L180" s="9" t="n"/>
       <c r="M180" s="9" t="n"/>
       <c r="N180" s="11" t="n"/>
+      <c r="O180" s="11">
+        <f>IF(D180="","",IF(COUNTIFS($A$5:$A$404,A180,$D$5:$D$404,D180,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A180,$D$5:$D$404,D180,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="11" t="n"/>
@@ -4185,6 +4895,10 @@
       <c r="L181" s="9" t="n"/>
       <c r="M181" s="9" t="n"/>
       <c r="N181" s="11" t="n"/>
+      <c r="O181" s="11">
+        <f>IF(D181="","",IF(COUNTIFS($A$5:$A$404,A181,$D$5:$D$404,D181,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A181,$D$5:$D$404,D181,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="11" t="n"/>
@@ -4204,6 +4918,10 @@
       <c r="L182" s="9" t="n"/>
       <c r="M182" s="9" t="n"/>
       <c r="N182" s="11" t="n"/>
+      <c r="O182" s="11">
+        <f>IF(D182="","",IF(COUNTIFS($A$5:$A$404,A182,$D$5:$D$404,D182,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A182,$D$5:$D$404,D182,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="11" t="n"/>
@@ -4223,6 +4941,10 @@
       <c r="L183" s="9" t="n"/>
       <c r="M183" s="9" t="n"/>
       <c r="N183" s="11" t="n"/>
+      <c r="O183" s="11">
+        <f>IF(D183="","",IF(COUNTIFS($A$5:$A$404,A183,$D$5:$D$404,D183,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A183,$D$5:$D$404,D183,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="11" t="n"/>
@@ -4242,6 +4964,10 @@
       <c r="L184" s="9" t="n"/>
       <c r="M184" s="9" t="n"/>
       <c r="N184" s="11" t="n"/>
+      <c r="O184" s="11">
+        <f>IF(D184="","",IF(COUNTIFS($A$5:$A$404,A184,$D$5:$D$404,D184,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A184,$D$5:$D$404,D184,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="11" t="n"/>
@@ -4261,6 +4987,10 @@
       <c r="L185" s="9" t="n"/>
       <c r="M185" s="9" t="n"/>
       <c r="N185" s="11" t="n"/>
+      <c r="O185" s="11">
+        <f>IF(D185="","",IF(COUNTIFS($A$5:$A$404,A185,$D$5:$D$404,D185,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A185,$D$5:$D$404,D185,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="11" t="n"/>
@@ -4280,6 +5010,10 @@
       <c r="L186" s="9" t="n"/>
       <c r="M186" s="9" t="n"/>
       <c r="N186" s="11" t="n"/>
+      <c r="O186" s="11">
+        <f>IF(D186="","",IF(COUNTIFS($A$5:$A$404,A186,$D$5:$D$404,D186,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A186,$D$5:$D$404,D186,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="11" t="n"/>
@@ -4299,6 +5033,10 @@
       <c r="L187" s="9" t="n"/>
       <c r="M187" s="9" t="n"/>
       <c r="N187" s="11" t="n"/>
+      <c r="O187" s="11">
+        <f>IF(D187="","",IF(COUNTIFS($A$5:$A$404,A187,$D$5:$D$404,D187,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A187,$D$5:$D$404,D187,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="11" t="n"/>
@@ -4318,6 +5056,10 @@
       <c r="L188" s="9" t="n"/>
       <c r="M188" s="9" t="n"/>
       <c r="N188" s="11" t="n"/>
+      <c r="O188" s="11">
+        <f>IF(D188="","",IF(COUNTIFS($A$5:$A$404,A188,$D$5:$D$404,D188,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A188,$D$5:$D$404,D188,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="11" t="n"/>
@@ -4337,6 +5079,10 @@
       <c r="L189" s="9" t="n"/>
       <c r="M189" s="9" t="n"/>
       <c r="N189" s="11" t="n"/>
+      <c r="O189" s="11">
+        <f>IF(D189="","",IF(COUNTIFS($A$5:$A$404,A189,$D$5:$D$404,D189,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A189,$D$5:$D$404,D189,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="11" t="n"/>
@@ -4356,6 +5102,10 @@
       <c r="L190" s="9" t="n"/>
       <c r="M190" s="9" t="n"/>
       <c r="N190" s="11" t="n"/>
+      <c r="O190" s="11">
+        <f>IF(D190="","",IF(COUNTIFS($A$5:$A$404,A190,$D$5:$D$404,D190,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A190,$D$5:$D$404,D190,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="11" t="n"/>
@@ -4375,6 +5125,10 @@
       <c r="L191" s="9" t="n"/>
       <c r="M191" s="9" t="n"/>
       <c r="N191" s="11" t="n"/>
+      <c r="O191" s="11">
+        <f>IF(D191="","",IF(COUNTIFS($A$5:$A$404,A191,$D$5:$D$404,D191,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A191,$D$5:$D$404,D191,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="11" t="n"/>
@@ -4394,6 +5148,10 @@
       <c r="L192" s="9" t="n"/>
       <c r="M192" s="9" t="n"/>
       <c r="N192" s="11" t="n"/>
+      <c r="O192" s="11">
+        <f>IF(D192="","",IF(COUNTIFS($A$5:$A$404,A192,$D$5:$D$404,D192,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A192,$D$5:$D$404,D192,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="11" t="n"/>
@@ -4413,6 +5171,10 @@
       <c r="L193" s="9" t="n"/>
       <c r="M193" s="9" t="n"/>
       <c r="N193" s="11" t="n"/>
+      <c r="O193" s="11">
+        <f>IF(D193="","",IF(COUNTIFS($A$5:$A$404,A193,$D$5:$D$404,D193,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A193,$D$5:$D$404,D193,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="11" t="n"/>
@@ -4432,6 +5194,10 @@
       <c r="L194" s="9" t="n"/>
       <c r="M194" s="9" t="n"/>
       <c r="N194" s="11" t="n"/>
+      <c r="O194" s="11">
+        <f>IF(D194="","",IF(COUNTIFS($A$5:$A$404,A194,$D$5:$D$404,D194,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A194,$D$5:$D$404,D194,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="11" t="n"/>
@@ -4451,6 +5217,10 @@
       <c r="L195" s="9" t="n"/>
       <c r="M195" s="9" t="n"/>
       <c r="N195" s="11" t="n"/>
+      <c r="O195" s="11">
+        <f>IF(D195="","",IF(COUNTIFS($A$5:$A$404,A195,$D$5:$D$404,D195,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A195,$D$5:$D$404,D195,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="11" t="n"/>
@@ -4470,6 +5240,10 @@
       <c r="L196" s="9" t="n"/>
       <c r="M196" s="9" t="n"/>
       <c r="N196" s="11" t="n"/>
+      <c r="O196" s="11">
+        <f>IF(D196="","",IF(COUNTIFS($A$5:$A$404,A196,$D$5:$D$404,D196,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A196,$D$5:$D$404,D196,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="11" t="n"/>
@@ -4489,6 +5263,10 @@
       <c r="L197" s="9" t="n"/>
       <c r="M197" s="9" t="n"/>
       <c r="N197" s="11" t="n"/>
+      <c r="O197" s="11">
+        <f>IF(D197="","",IF(COUNTIFS($A$5:$A$404,A197,$D$5:$D$404,D197,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A197,$D$5:$D$404,D197,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="11" t="n"/>
@@ -4508,6 +5286,10 @@
       <c r="L198" s="9" t="n"/>
       <c r="M198" s="9" t="n"/>
       <c r="N198" s="11" t="n"/>
+      <c r="O198" s="11">
+        <f>IF(D198="","",IF(COUNTIFS($A$5:$A$404,A198,$D$5:$D$404,D198,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A198,$D$5:$D$404,D198,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="11" t="n"/>
@@ -4527,6 +5309,10 @@
       <c r="L199" s="9" t="n"/>
       <c r="M199" s="9" t="n"/>
       <c r="N199" s="11" t="n"/>
+      <c r="O199" s="11">
+        <f>IF(D199="","",IF(COUNTIFS($A$5:$A$404,A199,$D$5:$D$404,D199,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A199,$D$5:$D$404,D199,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="11" t="n"/>
@@ -4546,6 +5332,10 @@
       <c r="L200" s="9" t="n"/>
       <c r="M200" s="9" t="n"/>
       <c r="N200" s="11" t="n"/>
+      <c r="O200" s="11">
+        <f>IF(D200="","",IF(COUNTIFS($A$5:$A$404,A200,$D$5:$D$404,D200,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A200,$D$5:$D$404,D200,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="11" t="n"/>
@@ -4565,6 +5355,10 @@
       <c r="L201" s="9" t="n"/>
       <c r="M201" s="9" t="n"/>
       <c r="N201" s="11" t="n"/>
+      <c r="O201" s="11">
+        <f>IF(D201="","",IF(COUNTIFS($A$5:$A$404,A201,$D$5:$D$404,D201,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A201,$D$5:$D$404,D201,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="11" t="n"/>
@@ -4584,6 +5378,10 @@
       <c r="L202" s="9" t="n"/>
       <c r="M202" s="9" t="n"/>
       <c r="N202" s="11" t="n"/>
+      <c r="O202" s="11">
+        <f>IF(D202="","",IF(COUNTIFS($A$5:$A$404,A202,$D$5:$D$404,D202,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A202,$D$5:$D$404,D202,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="11" t="n"/>
@@ -4603,6 +5401,10 @@
       <c r="L203" s="9" t="n"/>
       <c r="M203" s="9" t="n"/>
       <c r="N203" s="11" t="n"/>
+      <c r="O203" s="11">
+        <f>IF(D203="","",IF(COUNTIFS($A$5:$A$404,A203,$D$5:$D$404,D203,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A203,$D$5:$D$404,D203,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="11" t="n"/>
@@ -4622,6 +5424,10 @@
       <c r="L204" s="9" t="n"/>
       <c r="M204" s="9" t="n"/>
       <c r="N204" s="11" t="n"/>
+      <c r="O204" s="11">
+        <f>IF(D204="","",IF(COUNTIFS($A$5:$A$404,A204,$D$5:$D$404,D204,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A204,$D$5:$D$404,D204,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="11" t="n"/>
@@ -4641,6 +5447,10 @@
       <c r="L205" s="9" t="n"/>
       <c r="M205" s="9" t="n"/>
       <c r="N205" s="11" t="n"/>
+      <c r="O205" s="11">
+        <f>IF(D205="","",IF(COUNTIFS($A$5:$A$404,A205,$D$5:$D$404,D205,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A205,$D$5:$D$404,D205,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="11" t="n"/>
@@ -4660,6 +5470,10 @@
       <c r="L206" s="9" t="n"/>
       <c r="M206" s="9" t="n"/>
       <c r="N206" s="11" t="n"/>
+      <c r="O206" s="11">
+        <f>IF(D206="","",IF(COUNTIFS($A$5:$A$404,A206,$D$5:$D$404,D206,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A206,$D$5:$D$404,D206,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="11" t="n"/>
@@ -4679,6 +5493,10 @@
       <c r="L207" s="9" t="n"/>
       <c r="M207" s="9" t="n"/>
       <c r="N207" s="11" t="n"/>
+      <c r="O207" s="11">
+        <f>IF(D207="","",IF(COUNTIFS($A$5:$A$404,A207,$D$5:$D$404,D207,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A207,$D$5:$D$404,D207,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="11" t="n"/>
@@ -4698,6 +5516,10 @@
       <c r="L208" s="9" t="n"/>
       <c r="M208" s="9" t="n"/>
       <c r="N208" s="11" t="n"/>
+      <c r="O208" s="11">
+        <f>IF(D208="","",IF(COUNTIFS($A$5:$A$404,A208,$D$5:$D$404,D208,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A208,$D$5:$D$404,D208,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="11" t="n"/>
@@ -4717,6 +5539,10 @@
       <c r="L209" s="9" t="n"/>
       <c r="M209" s="9" t="n"/>
       <c r="N209" s="11" t="n"/>
+      <c r="O209" s="11">
+        <f>IF(D209="","",IF(COUNTIFS($A$5:$A$404,A209,$D$5:$D$404,D209,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A209,$D$5:$D$404,D209,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="11" t="n"/>
@@ -4736,6 +5562,10 @@
       <c r="L210" s="9" t="n"/>
       <c r="M210" s="9" t="n"/>
       <c r="N210" s="11" t="n"/>
+      <c r="O210" s="11">
+        <f>IF(D210="","",IF(COUNTIFS($A$5:$A$404,A210,$D$5:$D$404,D210,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A210,$D$5:$D$404,D210,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="11" t="n"/>
@@ -4755,6 +5585,10 @@
       <c r="L211" s="9" t="n"/>
       <c r="M211" s="9" t="n"/>
       <c r="N211" s="11" t="n"/>
+      <c r="O211" s="11">
+        <f>IF(D211="","",IF(COUNTIFS($A$5:$A$404,A211,$D$5:$D$404,D211,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A211,$D$5:$D$404,D211,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="11" t="n"/>
@@ -4774,6 +5608,10 @@
       <c r="L212" s="9" t="n"/>
       <c r="M212" s="9" t="n"/>
       <c r="N212" s="11" t="n"/>
+      <c r="O212" s="11">
+        <f>IF(D212="","",IF(COUNTIFS($A$5:$A$404,A212,$D$5:$D$404,D212,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A212,$D$5:$D$404,D212,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="11" t="n"/>
@@ -4793,6 +5631,10 @@
       <c r="L213" s="9" t="n"/>
       <c r="M213" s="9" t="n"/>
       <c r="N213" s="11" t="n"/>
+      <c r="O213" s="11">
+        <f>IF(D213="","",IF(COUNTIFS($A$5:$A$404,A213,$D$5:$D$404,D213,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A213,$D$5:$D$404,D213,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="11" t="n"/>
@@ -4812,6 +5654,10 @@
       <c r="L214" s="9" t="n"/>
       <c r="M214" s="9" t="n"/>
       <c r="N214" s="11" t="n"/>
+      <c r="O214" s="11">
+        <f>IF(D214="","",IF(COUNTIFS($A$5:$A$404,A214,$D$5:$D$404,D214,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A214,$D$5:$D$404,D214,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="11" t="n"/>
@@ -4831,6 +5677,10 @@
       <c r="L215" s="9" t="n"/>
       <c r="M215" s="9" t="n"/>
       <c r="N215" s="11" t="n"/>
+      <c r="O215" s="11">
+        <f>IF(D215="","",IF(COUNTIFS($A$5:$A$404,A215,$D$5:$D$404,D215,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A215,$D$5:$D$404,D215,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="11" t="n"/>
@@ -4850,6 +5700,10 @@
       <c r="L216" s="9" t="n"/>
       <c r="M216" s="9" t="n"/>
       <c r="N216" s="11" t="n"/>
+      <c r="O216" s="11">
+        <f>IF(D216="","",IF(COUNTIFS($A$5:$A$404,A216,$D$5:$D$404,D216,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A216,$D$5:$D$404,D216,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="11" t="n"/>
@@ -4869,6 +5723,10 @@
       <c r="L217" s="9" t="n"/>
       <c r="M217" s="9" t="n"/>
       <c r="N217" s="11" t="n"/>
+      <c r="O217" s="11">
+        <f>IF(D217="","",IF(COUNTIFS($A$5:$A$404,A217,$D$5:$D$404,D217,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A217,$D$5:$D$404,D217,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="11" t="n"/>
@@ -4888,6 +5746,10 @@
       <c r="L218" s="9" t="n"/>
       <c r="M218" s="9" t="n"/>
       <c r="N218" s="11" t="n"/>
+      <c r="O218" s="11">
+        <f>IF(D218="","",IF(COUNTIFS($A$5:$A$404,A218,$D$5:$D$404,D218,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A218,$D$5:$D$404,D218,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="11" t="n"/>
@@ -4907,6 +5769,10 @@
       <c r="L219" s="9" t="n"/>
       <c r="M219" s="9" t="n"/>
       <c r="N219" s="11" t="n"/>
+      <c r="O219" s="11">
+        <f>IF(D219="","",IF(COUNTIFS($A$5:$A$404,A219,$D$5:$D$404,D219,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A219,$D$5:$D$404,D219,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="11" t="n"/>
@@ -4926,6 +5792,10 @@
       <c r="L220" s="9" t="n"/>
       <c r="M220" s="9" t="n"/>
       <c r="N220" s="11" t="n"/>
+      <c r="O220" s="11">
+        <f>IF(D220="","",IF(COUNTIFS($A$5:$A$404,A220,$D$5:$D$404,D220,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A220,$D$5:$D$404,D220,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="11" t="n"/>
@@ -4945,6 +5815,10 @@
       <c r="L221" s="9" t="n"/>
       <c r="M221" s="9" t="n"/>
       <c r="N221" s="11" t="n"/>
+      <c r="O221" s="11">
+        <f>IF(D221="","",IF(COUNTIFS($A$5:$A$404,A221,$D$5:$D$404,D221,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A221,$D$5:$D$404,D221,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="11" t="n"/>
@@ -4964,6 +5838,10 @@
       <c r="L222" s="9" t="n"/>
       <c r="M222" s="9" t="n"/>
       <c r="N222" s="11" t="n"/>
+      <c r="O222" s="11">
+        <f>IF(D222="","",IF(COUNTIFS($A$5:$A$404,A222,$D$5:$D$404,D222,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A222,$D$5:$D$404,D222,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="11" t="n"/>
@@ -4983,6 +5861,10 @@
       <c r="L223" s="9" t="n"/>
       <c r="M223" s="9" t="n"/>
       <c r="N223" s="11" t="n"/>
+      <c r="O223" s="11">
+        <f>IF(D223="","",IF(COUNTIFS($A$5:$A$404,A223,$D$5:$D$404,D223,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A223,$D$5:$D$404,D223,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="11" t="n"/>
@@ -5002,6 +5884,10 @@
       <c r="L224" s="9" t="n"/>
       <c r="M224" s="9" t="n"/>
       <c r="N224" s="11" t="n"/>
+      <c r="O224" s="11">
+        <f>IF(D224="","",IF(COUNTIFS($A$5:$A$404,A224,$D$5:$D$404,D224,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A224,$D$5:$D$404,D224,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="11" t="n"/>
@@ -5021,6 +5907,10 @@
       <c r="L225" s="9" t="n"/>
       <c r="M225" s="9" t="n"/>
       <c r="N225" s="11" t="n"/>
+      <c r="O225" s="11">
+        <f>IF(D225="","",IF(COUNTIFS($A$5:$A$404,A225,$D$5:$D$404,D225,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A225,$D$5:$D$404,D225,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="11" t="n"/>
@@ -5040,6 +5930,10 @@
       <c r="L226" s="9" t="n"/>
       <c r="M226" s="9" t="n"/>
       <c r="N226" s="11" t="n"/>
+      <c r="O226" s="11">
+        <f>IF(D226="","",IF(COUNTIFS($A$5:$A$404,A226,$D$5:$D$404,D226,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A226,$D$5:$D$404,D226,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="11" t="n"/>
@@ -5059,6 +5953,10 @@
       <c r="L227" s="9" t="n"/>
       <c r="M227" s="9" t="n"/>
       <c r="N227" s="11" t="n"/>
+      <c r="O227" s="11">
+        <f>IF(D227="","",IF(COUNTIFS($A$5:$A$404,A227,$D$5:$D$404,D227,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A227,$D$5:$D$404,D227,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="11" t="n"/>
@@ -5078,6 +5976,10 @@
       <c r="L228" s="9" t="n"/>
       <c r="M228" s="9" t="n"/>
       <c r="N228" s="11" t="n"/>
+      <c r="O228" s="11">
+        <f>IF(D228="","",IF(COUNTIFS($A$5:$A$404,A228,$D$5:$D$404,D228,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A228,$D$5:$D$404,D228,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="11" t="n"/>
@@ -5097,6 +5999,10 @@
       <c r="L229" s="9" t="n"/>
       <c r="M229" s="9" t="n"/>
       <c r="N229" s="11" t="n"/>
+      <c r="O229" s="11">
+        <f>IF(D229="","",IF(COUNTIFS($A$5:$A$404,A229,$D$5:$D$404,D229,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A229,$D$5:$D$404,D229,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="11" t="n"/>
@@ -5116,6 +6022,10 @@
       <c r="L230" s="9" t="n"/>
       <c r="M230" s="9" t="n"/>
       <c r="N230" s="11" t="n"/>
+      <c r="O230" s="11">
+        <f>IF(D230="","",IF(COUNTIFS($A$5:$A$404,A230,$D$5:$D$404,D230,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A230,$D$5:$D$404,D230,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="11" t="n"/>
@@ -5135,6 +6045,10 @@
       <c r="L231" s="9" t="n"/>
       <c r="M231" s="9" t="n"/>
       <c r="N231" s="11" t="n"/>
+      <c r="O231" s="11">
+        <f>IF(D231="","",IF(COUNTIFS($A$5:$A$404,A231,$D$5:$D$404,D231,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A231,$D$5:$D$404,D231,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="11" t="n"/>
@@ -5154,6 +6068,10 @@
       <c r="L232" s="9" t="n"/>
       <c r="M232" s="9" t="n"/>
       <c r="N232" s="11" t="n"/>
+      <c r="O232" s="11">
+        <f>IF(D232="","",IF(COUNTIFS($A$5:$A$404,A232,$D$5:$D$404,D232,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A232,$D$5:$D$404,D232,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="11" t="n"/>
@@ -5173,6 +6091,10 @@
       <c r="L233" s="9" t="n"/>
       <c r="M233" s="9" t="n"/>
       <c r="N233" s="11" t="n"/>
+      <c r="O233" s="11">
+        <f>IF(D233="","",IF(COUNTIFS($A$5:$A$404,A233,$D$5:$D$404,D233,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A233,$D$5:$D$404,D233,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="11" t="n"/>
@@ -5192,6 +6114,10 @@
       <c r="L234" s="9" t="n"/>
       <c r="M234" s="9" t="n"/>
       <c r="N234" s="11" t="n"/>
+      <c r="O234" s="11">
+        <f>IF(D234="","",IF(COUNTIFS($A$5:$A$404,A234,$D$5:$D$404,D234,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A234,$D$5:$D$404,D234,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="11" t="n"/>
@@ -5211,6 +6137,10 @@
       <c r="L235" s="9" t="n"/>
       <c r="M235" s="9" t="n"/>
       <c r="N235" s="11" t="n"/>
+      <c r="O235" s="11">
+        <f>IF(D235="","",IF(COUNTIFS($A$5:$A$404,A235,$D$5:$D$404,D235,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A235,$D$5:$D$404,D235,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="11" t="n"/>
@@ -5230,6 +6160,10 @@
       <c r="L236" s="9" t="n"/>
       <c r="M236" s="9" t="n"/>
       <c r="N236" s="11" t="n"/>
+      <c r="O236" s="11">
+        <f>IF(D236="","",IF(COUNTIFS($A$5:$A$404,A236,$D$5:$D$404,D236,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A236,$D$5:$D$404,D236,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="11" t="n"/>
@@ -5249,6 +6183,10 @@
       <c r="L237" s="9" t="n"/>
       <c r="M237" s="9" t="n"/>
       <c r="N237" s="11" t="n"/>
+      <c r="O237" s="11">
+        <f>IF(D237="","",IF(COUNTIFS($A$5:$A$404,A237,$D$5:$D$404,D237,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A237,$D$5:$D$404,D237,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="11" t="n"/>
@@ -5268,6 +6206,10 @@
       <c r="L238" s="9" t="n"/>
       <c r="M238" s="9" t="n"/>
       <c r="N238" s="11" t="n"/>
+      <c r="O238" s="11">
+        <f>IF(D238="","",IF(COUNTIFS($A$5:$A$404,A238,$D$5:$D$404,D238,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A238,$D$5:$D$404,D238,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="11" t="n"/>
@@ -5287,6 +6229,10 @@
       <c r="L239" s="9" t="n"/>
       <c r="M239" s="9" t="n"/>
       <c r="N239" s="11" t="n"/>
+      <c r="O239" s="11">
+        <f>IF(D239="","",IF(COUNTIFS($A$5:$A$404,A239,$D$5:$D$404,D239,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A239,$D$5:$D$404,D239,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="11" t="n"/>
@@ -5306,6 +6252,10 @@
       <c r="L240" s="9" t="n"/>
       <c r="M240" s="9" t="n"/>
       <c r="N240" s="11" t="n"/>
+      <c r="O240" s="11">
+        <f>IF(D240="","",IF(COUNTIFS($A$5:$A$404,A240,$D$5:$D$404,D240,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A240,$D$5:$D$404,D240,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="11" t="n"/>
@@ -5325,6 +6275,10 @@
       <c r="L241" s="9" t="n"/>
       <c r="M241" s="9" t="n"/>
       <c r="N241" s="11" t="n"/>
+      <c r="O241" s="11">
+        <f>IF(D241="","",IF(COUNTIFS($A$5:$A$404,A241,$D$5:$D$404,D241,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A241,$D$5:$D$404,D241,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="11" t="n"/>
@@ -5344,6 +6298,10 @@
       <c r="L242" s="9" t="n"/>
       <c r="M242" s="9" t="n"/>
       <c r="N242" s="11" t="n"/>
+      <c r="O242" s="11">
+        <f>IF(D242="","",IF(COUNTIFS($A$5:$A$404,A242,$D$5:$D$404,D242,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A242,$D$5:$D$404,D242,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="11" t="n"/>
@@ -5363,6 +6321,10 @@
       <c r="L243" s="9" t="n"/>
       <c r="M243" s="9" t="n"/>
       <c r="N243" s="11" t="n"/>
+      <c r="O243" s="11">
+        <f>IF(D243="","",IF(COUNTIFS($A$5:$A$404,A243,$D$5:$D$404,D243,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A243,$D$5:$D$404,D243,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="11" t="n"/>
@@ -5382,6 +6344,10 @@
       <c r="L244" s="9" t="n"/>
       <c r="M244" s="9" t="n"/>
       <c r="N244" s="11" t="n"/>
+      <c r="O244" s="11">
+        <f>IF(D244="","",IF(COUNTIFS($A$5:$A$404,A244,$D$5:$D$404,D244,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A244,$D$5:$D$404,D244,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="11" t="n"/>
@@ -5401,6 +6367,10 @@
       <c r="L245" s="9" t="n"/>
       <c r="M245" s="9" t="n"/>
       <c r="N245" s="11" t="n"/>
+      <c r="O245" s="11">
+        <f>IF(D245="","",IF(COUNTIFS($A$5:$A$404,A245,$D$5:$D$404,D245,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A245,$D$5:$D$404,D245,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="11" t="n"/>
@@ -5420,6 +6390,10 @@
       <c r="L246" s="9" t="n"/>
       <c r="M246" s="9" t="n"/>
       <c r="N246" s="11" t="n"/>
+      <c r="O246" s="11">
+        <f>IF(D246="","",IF(COUNTIFS($A$5:$A$404,A246,$D$5:$D$404,D246,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A246,$D$5:$D$404,D246,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="11" t="n"/>
@@ -5439,6 +6413,10 @@
       <c r="L247" s="9" t="n"/>
       <c r="M247" s="9" t="n"/>
       <c r="N247" s="11" t="n"/>
+      <c r="O247" s="11">
+        <f>IF(D247="","",IF(COUNTIFS($A$5:$A$404,A247,$D$5:$D$404,D247,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A247,$D$5:$D$404,D247,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="11" t="n"/>
@@ -5458,6 +6436,10 @@
       <c r="L248" s="9" t="n"/>
       <c r="M248" s="9" t="n"/>
       <c r="N248" s="11" t="n"/>
+      <c r="O248" s="11">
+        <f>IF(D248="","",IF(COUNTIFS($A$5:$A$404,A248,$D$5:$D$404,D248,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A248,$D$5:$D$404,D248,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="11" t="n"/>
@@ -5477,6 +6459,10 @@
       <c r="L249" s="9" t="n"/>
       <c r="M249" s="9" t="n"/>
       <c r="N249" s="11" t="n"/>
+      <c r="O249" s="11">
+        <f>IF(D249="","",IF(COUNTIFS($A$5:$A$404,A249,$D$5:$D$404,D249,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A249,$D$5:$D$404,D249,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="11" t="n"/>
@@ -5496,6 +6482,10 @@
       <c r="L250" s="9" t="n"/>
       <c r="M250" s="9" t="n"/>
       <c r="N250" s="11" t="n"/>
+      <c r="O250" s="11">
+        <f>IF(D250="","",IF(COUNTIFS($A$5:$A$404,A250,$D$5:$D$404,D250,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A250,$D$5:$D$404,D250,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="11" t="n"/>
@@ -5515,6 +6505,10 @@
       <c r="L251" s="9" t="n"/>
       <c r="M251" s="9" t="n"/>
       <c r="N251" s="11" t="n"/>
+      <c r="O251" s="11">
+        <f>IF(D251="","",IF(COUNTIFS($A$5:$A$404,A251,$D$5:$D$404,D251,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A251,$D$5:$D$404,D251,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="11" t="n"/>
@@ -5534,6 +6528,10 @@
       <c r="L252" s="9" t="n"/>
       <c r="M252" s="9" t="n"/>
       <c r="N252" s="11" t="n"/>
+      <c r="O252" s="11">
+        <f>IF(D252="","",IF(COUNTIFS($A$5:$A$404,A252,$D$5:$D$404,D252,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A252,$D$5:$D$404,D252,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="11" t="n"/>
@@ -5553,6 +6551,10 @@
       <c r="L253" s="9" t="n"/>
       <c r="M253" s="9" t="n"/>
       <c r="N253" s="11" t="n"/>
+      <c r="O253" s="11">
+        <f>IF(D253="","",IF(COUNTIFS($A$5:$A$404,A253,$D$5:$D$404,D253,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A253,$D$5:$D$404,D253,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="11" t="n"/>
@@ -5572,6 +6574,10 @@
       <c r="L254" s="9" t="n"/>
       <c r="M254" s="9" t="n"/>
       <c r="N254" s="11" t="n"/>
+      <c r="O254" s="11">
+        <f>IF(D254="","",IF(COUNTIFS($A$5:$A$404,A254,$D$5:$D$404,D254,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A254,$D$5:$D$404,D254,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="11" t="n"/>
@@ -5591,6 +6597,10 @@
       <c r="L255" s="9" t="n"/>
       <c r="M255" s="9" t="n"/>
       <c r="N255" s="11" t="n"/>
+      <c r="O255" s="11">
+        <f>IF(D255="","",IF(COUNTIFS($A$5:$A$404,A255,$D$5:$D$404,D255,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A255,$D$5:$D$404,D255,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="11" t="n"/>
@@ -5610,6 +6620,10 @@
       <c r="L256" s="9" t="n"/>
       <c r="M256" s="9" t="n"/>
       <c r="N256" s="11" t="n"/>
+      <c r="O256" s="11">
+        <f>IF(D256="","",IF(COUNTIFS($A$5:$A$404,A256,$D$5:$D$404,D256,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A256,$D$5:$D$404,D256,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="11" t="n"/>
@@ -5629,6 +6643,10 @@
       <c r="L257" s="9" t="n"/>
       <c r="M257" s="9" t="n"/>
       <c r="N257" s="11" t="n"/>
+      <c r="O257" s="11">
+        <f>IF(D257="","",IF(COUNTIFS($A$5:$A$404,A257,$D$5:$D$404,D257,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A257,$D$5:$D$404,D257,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="11" t="n"/>
@@ -5648,6 +6666,10 @@
       <c r="L258" s="9" t="n"/>
       <c r="M258" s="9" t="n"/>
       <c r="N258" s="11" t="n"/>
+      <c r="O258" s="11">
+        <f>IF(D258="","",IF(COUNTIFS($A$5:$A$404,A258,$D$5:$D$404,D258,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A258,$D$5:$D$404,D258,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="11" t="n"/>
@@ -5667,6 +6689,10 @@
       <c r="L259" s="9" t="n"/>
       <c r="M259" s="9" t="n"/>
       <c r="N259" s="11" t="n"/>
+      <c r="O259" s="11">
+        <f>IF(D259="","",IF(COUNTIFS($A$5:$A$404,A259,$D$5:$D$404,D259,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A259,$D$5:$D$404,D259,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="11" t="n"/>
@@ -5686,6 +6712,10 @@
       <c r="L260" s="9" t="n"/>
       <c r="M260" s="9" t="n"/>
       <c r="N260" s="11" t="n"/>
+      <c r="O260" s="11">
+        <f>IF(D260="","",IF(COUNTIFS($A$5:$A$404,A260,$D$5:$D$404,D260,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A260,$D$5:$D$404,D260,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="11" t="n"/>
@@ -5705,6 +6735,10 @@
       <c r="L261" s="9" t="n"/>
       <c r="M261" s="9" t="n"/>
       <c r="N261" s="11" t="n"/>
+      <c r="O261" s="11">
+        <f>IF(D261="","",IF(COUNTIFS($A$5:$A$404,A261,$D$5:$D$404,D261,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A261,$D$5:$D$404,D261,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="11" t="n"/>
@@ -5724,6 +6758,10 @@
       <c r="L262" s="9" t="n"/>
       <c r="M262" s="9" t="n"/>
       <c r="N262" s="11" t="n"/>
+      <c r="O262" s="11">
+        <f>IF(D262="","",IF(COUNTIFS($A$5:$A$404,A262,$D$5:$D$404,D262,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A262,$D$5:$D$404,D262,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="11" t="n"/>
@@ -5743,6 +6781,10 @@
       <c r="L263" s="9" t="n"/>
       <c r="M263" s="9" t="n"/>
       <c r="N263" s="11" t="n"/>
+      <c r="O263" s="11">
+        <f>IF(D263="","",IF(COUNTIFS($A$5:$A$404,A263,$D$5:$D$404,D263,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A263,$D$5:$D$404,D263,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="11" t="n"/>
@@ -5762,6 +6804,10 @@
       <c r="L264" s="9" t="n"/>
       <c r="M264" s="9" t="n"/>
       <c r="N264" s="11" t="n"/>
+      <c r="O264" s="11">
+        <f>IF(D264="","",IF(COUNTIFS($A$5:$A$404,A264,$D$5:$D$404,D264,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A264,$D$5:$D$404,D264,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="11" t="n"/>
@@ -5781,6 +6827,10 @@
       <c r="L265" s="9" t="n"/>
       <c r="M265" s="9" t="n"/>
       <c r="N265" s="11" t="n"/>
+      <c r="O265" s="11">
+        <f>IF(D265="","",IF(COUNTIFS($A$5:$A$404,A265,$D$5:$D$404,D265,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A265,$D$5:$D$404,D265,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="11" t="n"/>
@@ -5800,6 +6850,10 @@
       <c r="L266" s="9" t="n"/>
       <c r="M266" s="9" t="n"/>
       <c r="N266" s="11" t="n"/>
+      <c r="O266" s="11">
+        <f>IF(D266="","",IF(COUNTIFS($A$5:$A$404,A266,$D$5:$D$404,D266,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A266,$D$5:$D$404,D266,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="11" t="n"/>
@@ -5819,6 +6873,10 @@
       <c r="L267" s="9" t="n"/>
       <c r="M267" s="9" t="n"/>
       <c r="N267" s="11" t="n"/>
+      <c r="O267" s="11">
+        <f>IF(D267="","",IF(COUNTIFS($A$5:$A$404,A267,$D$5:$D$404,D267,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A267,$D$5:$D$404,D267,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="11" t="n"/>
@@ -5838,6 +6896,10 @@
       <c r="L268" s="9" t="n"/>
       <c r="M268" s="9" t="n"/>
       <c r="N268" s="11" t="n"/>
+      <c r="O268" s="11">
+        <f>IF(D268="","",IF(COUNTIFS($A$5:$A$404,A268,$D$5:$D$404,D268,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A268,$D$5:$D$404,D268,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="11" t="n"/>
@@ -5857,6 +6919,10 @@
       <c r="L269" s="9" t="n"/>
       <c r="M269" s="9" t="n"/>
       <c r="N269" s="11" t="n"/>
+      <c r="O269" s="11">
+        <f>IF(D269="","",IF(COUNTIFS($A$5:$A$404,A269,$D$5:$D$404,D269,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A269,$D$5:$D$404,D269,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="11" t="n"/>
@@ -5876,6 +6942,10 @@
       <c r="L270" s="9" t="n"/>
       <c r="M270" s="9" t="n"/>
       <c r="N270" s="11" t="n"/>
+      <c r="O270" s="11">
+        <f>IF(D270="","",IF(COUNTIFS($A$5:$A$404,A270,$D$5:$D$404,D270,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A270,$D$5:$D$404,D270,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="11" t="n"/>
@@ -5895,6 +6965,10 @@
       <c r="L271" s="9" t="n"/>
       <c r="M271" s="9" t="n"/>
       <c r="N271" s="11" t="n"/>
+      <c r="O271" s="11">
+        <f>IF(D271="","",IF(COUNTIFS($A$5:$A$404,A271,$D$5:$D$404,D271,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A271,$D$5:$D$404,D271,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="11" t="n"/>
@@ -5914,6 +6988,10 @@
       <c r="L272" s="9" t="n"/>
       <c r="M272" s="9" t="n"/>
       <c r="N272" s="11" t="n"/>
+      <c r="O272" s="11">
+        <f>IF(D272="","",IF(COUNTIFS($A$5:$A$404,A272,$D$5:$D$404,D272,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A272,$D$5:$D$404,D272,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="11" t="n"/>
@@ -5933,6 +7011,10 @@
       <c r="L273" s="9" t="n"/>
       <c r="M273" s="9" t="n"/>
       <c r="N273" s="11" t="n"/>
+      <c r="O273" s="11">
+        <f>IF(D273="","",IF(COUNTIFS($A$5:$A$404,A273,$D$5:$D$404,D273,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A273,$D$5:$D$404,D273,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="11" t="n"/>
@@ -5952,6 +7034,10 @@
       <c r="L274" s="9" t="n"/>
       <c r="M274" s="9" t="n"/>
       <c r="N274" s="11" t="n"/>
+      <c r="O274" s="11">
+        <f>IF(D274="","",IF(COUNTIFS($A$5:$A$404,A274,$D$5:$D$404,D274,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A274,$D$5:$D$404,D274,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="11" t="n"/>
@@ -5971,6 +7057,10 @@
       <c r="L275" s="9" t="n"/>
       <c r="M275" s="9" t="n"/>
       <c r="N275" s="11" t="n"/>
+      <c r="O275" s="11">
+        <f>IF(D275="","",IF(COUNTIFS($A$5:$A$404,A275,$D$5:$D$404,D275,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A275,$D$5:$D$404,D275,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="11" t="n"/>
@@ -5990,6 +7080,10 @@
       <c r="L276" s="9" t="n"/>
       <c r="M276" s="9" t="n"/>
       <c r="N276" s="11" t="n"/>
+      <c r="O276" s="11">
+        <f>IF(D276="","",IF(COUNTIFS($A$5:$A$404,A276,$D$5:$D$404,D276,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A276,$D$5:$D$404,D276,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="11" t="n"/>
@@ -6009,6 +7103,10 @@
       <c r="L277" s="9" t="n"/>
       <c r="M277" s="9" t="n"/>
       <c r="N277" s="11" t="n"/>
+      <c r="O277" s="11">
+        <f>IF(D277="","",IF(COUNTIFS($A$5:$A$404,A277,$D$5:$D$404,D277,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A277,$D$5:$D$404,D277,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="11" t="n"/>
@@ -6028,6 +7126,10 @@
       <c r="L278" s="9" t="n"/>
       <c r="M278" s="9" t="n"/>
       <c r="N278" s="11" t="n"/>
+      <c r="O278" s="11">
+        <f>IF(D278="","",IF(COUNTIFS($A$5:$A$404,A278,$D$5:$D$404,D278,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A278,$D$5:$D$404,D278,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="11" t="n"/>
@@ -6047,6 +7149,10 @@
       <c r="L279" s="9" t="n"/>
       <c r="M279" s="9" t="n"/>
       <c r="N279" s="11" t="n"/>
+      <c r="O279" s="11">
+        <f>IF(D279="","",IF(COUNTIFS($A$5:$A$404,A279,$D$5:$D$404,D279,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A279,$D$5:$D$404,D279,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="11" t="n"/>
@@ -6066,6 +7172,10 @@
       <c r="L280" s="9" t="n"/>
       <c r="M280" s="9" t="n"/>
       <c r="N280" s="11" t="n"/>
+      <c r="O280" s="11">
+        <f>IF(D280="","",IF(COUNTIFS($A$5:$A$404,A280,$D$5:$D$404,D280,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A280,$D$5:$D$404,D280,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="11" t="n"/>
@@ -6085,6 +7195,10 @@
       <c r="L281" s="9" t="n"/>
       <c r="M281" s="9" t="n"/>
       <c r="N281" s="11" t="n"/>
+      <c r="O281" s="11">
+        <f>IF(D281="","",IF(COUNTIFS($A$5:$A$404,A281,$D$5:$D$404,D281,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A281,$D$5:$D$404,D281,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="11" t="n"/>
@@ -6104,6 +7218,10 @@
       <c r="L282" s="9" t="n"/>
       <c r="M282" s="9" t="n"/>
       <c r="N282" s="11" t="n"/>
+      <c r="O282" s="11">
+        <f>IF(D282="","",IF(COUNTIFS($A$5:$A$404,A282,$D$5:$D$404,D282,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A282,$D$5:$D$404,D282,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="11" t="n"/>
@@ -6123,6 +7241,10 @@
       <c r="L283" s="9" t="n"/>
       <c r="M283" s="9" t="n"/>
       <c r="N283" s="11" t="n"/>
+      <c r="O283" s="11">
+        <f>IF(D283="","",IF(COUNTIFS($A$5:$A$404,A283,$D$5:$D$404,D283,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A283,$D$5:$D$404,D283,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="11" t="n"/>
@@ -6142,6 +7264,10 @@
       <c r="L284" s="9" t="n"/>
       <c r="M284" s="9" t="n"/>
       <c r="N284" s="11" t="n"/>
+      <c r="O284" s="11">
+        <f>IF(D284="","",IF(COUNTIFS($A$5:$A$404,A284,$D$5:$D$404,D284,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A284,$D$5:$D$404,D284,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="11" t="n"/>
@@ -6161,6 +7287,10 @@
       <c r="L285" s="9" t="n"/>
       <c r="M285" s="9" t="n"/>
       <c r="N285" s="11" t="n"/>
+      <c r="O285" s="11">
+        <f>IF(D285="","",IF(COUNTIFS($A$5:$A$404,A285,$D$5:$D$404,D285,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A285,$D$5:$D$404,D285,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="11" t="n"/>
@@ -6180,6 +7310,10 @@
       <c r="L286" s="9" t="n"/>
       <c r="M286" s="9" t="n"/>
       <c r="N286" s="11" t="n"/>
+      <c r="O286" s="11">
+        <f>IF(D286="","",IF(COUNTIFS($A$5:$A$404,A286,$D$5:$D$404,D286,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A286,$D$5:$D$404,D286,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="11" t="n"/>
@@ -6199,6 +7333,10 @@
       <c r="L287" s="9" t="n"/>
       <c r="M287" s="9" t="n"/>
       <c r="N287" s="11" t="n"/>
+      <c r="O287" s="11">
+        <f>IF(D287="","",IF(COUNTIFS($A$5:$A$404,A287,$D$5:$D$404,D287,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A287,$D$5:$D$404,D287,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="11" t="n"/>
@@ -6218,6 +7356,10 @@
       <c r="L288" s="9" t="n"/>
       <c r="M288" s="9" t="n"/>
       <c r="N288" s="11" t="n"/>
+      <c r="O288" s="11">
+        <f>IF(D288="","",IF(COUNTIFS($A$5:$A$404,A288,$D$5:$D$404,D288,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A288,$D$5:$D$404,D288,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="11" t="n"/>
@@ -6237,6 +7379,10 @@
       <c r="L289" s="9" t="n"/>
       <c r="M289" s="9" t="n"/>
       <c r="N289" s="11" t="n"/>
+      <c r="O289" s="11">
+        <f>IF(D289="","",IF(COUNTIFS($A$5:$A$404,A289,$D$5:$D$404,D289,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A289,$D$5:$D$404,D289,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="11" t="n"/>
@@ -6256,6 +7402,10 @@
       <c r="L290" s="9" t="n"/>
       <c r="M290" s="9" t="n"/>
       <c r="N290" s="11" t="n"/>
+      <c r="O290" s="11">
+        <f>IF(D290="","",IF(COUNTIFS($A$5:$A$404,A290,$D$5:$D$404,D290,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A290,$D$5:$D$404,D290,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="11" t="n"/>
@@ -6275,6 +7425,10 @@
       <c r="L291" s="9" t="n"/>
       <c r="M291" s="9" t="n"/>
       <c r="N291" s="11" t="n"/>
+      <c r="O291" s="11">
+        <f>IF(D291="","",IF(COUNTIFS($A$5:$A$404,A291,$D$5:$D$404,D291,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A291,$D$5:$D$404,D291,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="11" t="n"/>
@@ -6294,6 +7448,10 @@
       <c r="L292" s="9" t="n"/>
       <c r="M292" s="9" t="n"/>
       <c r="N292" s="11" t="n"/>
+      <c r="O292" s="11">
+        <f>IF(D292="","",IF(COUNTIFS($A$5:$A$404,A292,$D$5:$D$404,D292,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A292,$D$5:$D$404,D292,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="11" t="n"/>
@@ -6313,6 +7471,10 @@
       <c r="L293" s="9" t="n"/>
       <c r="M293" s="9" t="n"/>
       <c r="N293" s="11" t="n"/>
+      <c r="O293" s="11">
+        <f>IF(D293="","",IF(COUNTIFS($A$5:$A$404,A293,$D$5:$D$404,D293,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A293,$D$5:$D$404,D293,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="11" t="n"/>
@@ -6332,6 +7494,10 @@
       <c r="L294" s="9" t="n"/>
       <c r="M294" s="9" t="n"/>
       <c r="N294" s="11" t="n"/>
+      <c r="O294" s="11">
+        <f>IF(D294="","",IF(COUNTIFS($A$5:$A$404,A294,$D$5:$D$404,D294,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A294,$D$5:$D$404,D294,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="11" t="n"/>
@@ -6351,6 +7517,10 @@
       <c r="L295" s="9" t="n"/>
       <c r="M295" s="9" t="n"/>
       <c r="N295" s="11" t="n"/>
+      <c r="O295" s="11">
+        <f>IF(D295="","",IF(COUNTIFS($A$5:$A$404,A295,$D$5:$D$404,D295,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A295,$D$5:$D$404,D295,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="11" t="n"/>
@@ -6370,6 +7540,10 @@
       <c r="L296" s="9" t="n"/>
       <c r="M296" s="9" t="n"/>
       <c r="N296" s="11" t="n"/>
+      <c r="O296" s="11">
+        <f>IF(D296="","",IF(COUNTIFS($A$5:$A$404,A296,$D$5:$D$404,D296,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A296,$D$5:$D$404,D296,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="11" t="n"/>
@@ -6389,6 +7563,10 @@
       <c r="L297" s="9" t="n"/>
       <c r="M297" s="9" t="n"/>
       <c r="N297" s="11" t="n"/>
+      <c r="O297" s="11">
+        <f>IF(D297="","",IF(COUNTIFS($A$5:$A$404,A297,$D$5:$D$404,D297,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A297,$D$5:$D$404,D297,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="11" t="n"/>
@@ -6408,6 +7586,10 @@
       <c r="L298" s="9" t="n"/>
       <c r="M298" s="9" t="n"/>
       <c r="N298" s="11" t="n"/>
+      <c r="O298" s="11">
+        <f>IF(D298="","",IF(COUNTIFS($A$5:$A$404,A298,$D$5:$D$404,D298,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A298,$D$5:$D$404,D298,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="11" t="n"/>
@@ -6427,6 +7609,10 @@
       <c r="L299" s="9" t="n"/>
       <c r="M299" s="9" t="n"/>
       <c r="N299" s="11" t="n"/>
+      <c r="O299" s="11">
+        <f>IF(D299="","",IF(COUNTIFS($A$5:$A$404,A299,$D$5:$D$404,D299,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A299,$D$5:$D$404,D299,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="11" t="n"/>
@@ -6446,6 +7632,10 @@
       <c r="L300" s="9" t="n"/>
       <c r="M300" s="9" t="n"/>
       <c r="N300" s="11" t="n"/>
+      <c r="O300" s="11">
+        <f>IF(D300="","",IF(COUNTIFS($A$5:$A$404,A300,$D$5:$D$404,D300,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A300,$D$5:$D$404,D300,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="11" t="n"/>
@@ -6465,6 +7655,10 @@
       <c r="L301" s="9" t="n"/>
       <c r="M301" s="9" t="n"/>
       <c r="N301" s="11" t="n"/>
+      <c r="O301" s="11">
+        <f>IF(D301="","",IF(COUNTIFS($A$5:$A$404,A301,$D$5:$D$404,D301,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A301,$D$5:$D$404,D301,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="11" t="n"/>
@@ -6484,6 +7678,10 @@
       <c r="L302" s="9" t="n"/>
       <c r="M302" s="9" t="n"/>
       <c r="N302" s="11" t="n"/>
+      <c r="O302" s="11">
+        <f>IF(D302="","",IF(COUNTIFS($A$5:$A$404,A302,$D$5:$D$404,D302,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A302,$D$5:$D$404,D302,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="11" t="n"/>
@@ -6503,6 +7701,10 @@
       <c r="L303" s="9" t="n"/>
       <c r="M303" s="9" t="n"/>
       <c r="N303" s="11" t="n"/>
+      <c r="O303" s="11">
+        <f>IF(D303="","",IF(COUNTIFS($A$5:$A$404,A303,$D$5:$D$404,D303,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A303,$D$5:$D$404,D303,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="11" t="n"/>
@@ -6522,6 +7724,10 @@
       <c r="L304" s="9" t="n"/>
       <c r="M304" s="9" t="n"/>
       <c r="N304" s="11" t="n"/>
+      <c r="O304" s="11">
+        <f>IF(D304="","",IF(COUNTIFS($A$5:$A$404,A304,$D$5:$D$404,D304,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A304,$D$5:$D$404,D304,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="11" t="n"/>
@@ -6541,6 +7747,10 @@
       <c r="L305" s="9" t="n"/>
       <c r="M305" s="9" t="n"/>
       <c r="N305" s="11" t="n"/>
+      <c r="O305" s="11">
+        <f>IF(D305="","",IF(COUNTIFS($A$5:$A$404,A305,$D$5:$D$404,D305,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A305,$D$5:$D$404,D305,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="11" t="n"/>
@@ -6560,6 +7770,10 @@
       <c r="L306" s="9" t="n"/>
       <c r="M306" s="9" t="n"/>
       <c r="N306" s="11" t="n"/>
+      <c r="O306" s="11">
+        <f>IF(D306="","",IF(COUNTIFS($A$5:$A$404,A306,$D$5:$D$404,D306,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A306,$D$5:$D$404,D306,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="11" t="n"/>
@@ -6579,6 +7793,10 @@
       <c r="L307" s="9" t="n"/>
       <c r="M307" s="9" t="n"/>
       <c r="N307" s="11" t="n"/>
+      <c r="O307" s="11">
+        <f>IF(D307="","",IF(COUNTIFS($A$5:$A$404,A307,$D$5:$D$404,D307,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A307,$D$5:$D$404,D307,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="11" t="n"/>
@@ -6598,6 +7816,10 @@
       <c r="L308" s="9" t="n"/>
       <c r="M308" s="9" t="n"/>
       <c r="N308" s="11" t="n"/>
+      <c r="O308" s="11">
+        <f>IF(D308="","",IF(COUNTIFS($A$5:$A$404,A308,$D$5:$D$404,D308,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A308,$D$5:$D$404,D308,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="11" t="n"/>
@@ -6617,6 +7839,10 @@
       <c r="L309" s="9" t="n"/>
       <c r="M309" s="9" t="n"/>
       <c r="N309" s="11" t="n"/>
+      <c r="O309" s="11">
+        <f>IF(D309="","",IF(COUNTIFS($A$5:$A$404,A309,$D$5:$D$404,D309,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A309,$D$5:$D$404,D309,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="11" t="n"/>
@@ -6636,6 +7862,10 @@
       <c r="L310" s="9" t="n"/>
       <c r="M310" s="9" t="n"/>
       <c r="N310" s="11" t="n"/>
+      <c r="O310" s="11">
+        <f>IF(D310="","",IF(COUNTIFS($A$5:$A$404,A310,$D$5:$D$404,D310,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A310,$D$5:$D$404,D310,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="11" t="n"/>
@@ -6655,6 +7885,10 @@
       <c r="L311" s="9" t="n"/>
       <c r="M311" s="9" t="n"/>
       <c r="N311" s="11" t="n"/>
+      <c r="O311" s="11">
+        <f>IF(D311="","",IF(COUNTIFS($A$5:$A$404,A311,$D$5:$D$404,D311,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A311,$D$5:$D$404,D311,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="11" t="n"/>
@@ -6674,6 +7908,10 @@
       <c r="L312" s="9" t="n"/>
       <c r="M312" s="9" t="n"/>
       <c r="N312" s="11" t="n"/>
+      <c r="O312" s="11">
+        <f>IF(D312="","",IF(COUNTIFS($A$5:$A$404,A312,$D$5:$D$404,D312,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A312,$D$5:$D$404,D312,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="11" t="n"/>
@@ -6693,6 +7931,10 @@
       <c r="L313" s="9" t="n"/>
       <c r="M313" s="9" t="n"/>
       <c r="N313" s="11" t="n"/>
+      <c r="O313" s="11">
+        <f>IF(D313="","",IF(COUNTIFS($A$5:$A$404,A313,$D$5:$D$404,D313,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A313,$D$5:$D$404,D313,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="11" t="n"/>
@@ -6712,6 +7954,10 @@
       <c r="L314" s="9" t="n"/>
       <c r="M314" s="9" t="n"/>
       <c r="N314" s="11" t="n"/>
+      <c r="O314" s="11">
+        <f>IF(D314="","",IF(COUNTIFS($A$5:$A$404,A314,$D$5:$D$404,D314,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A314,$D$5:$D$404,D314,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="11" t="n"/>
@@ -6731,6 +7977,10 @@
       <c r="L315" s="9" t="n"/>
       <c r="M315" s="9" t="n"/>
       <c r="N315" s="11" t="n"/>
+      <c r="O315" s="11">
+        <f>IF(D315="","",IF(COUNTIFS($A$5:$A$404,A315,$D$5:$D$404,D315,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A315,$D$5:$D$404,D315,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="11" t="n"/>
@@ -6750,6 +8000,10 @@
       <c r="L316" s="9" t="n"/>
       <c r="M316" s="9" t="n"/>
       <c r="N316" s="11" t="n"/>
+      <c r="O316" s="11">
+        <f>IF(D316="","",IF(COUNTIFS($A$5:$A$404,A316,$D$5:$D$404,D316,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A316,$D$5:$D$404,D316,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="11" t="n"/>
@@ -6769,6 +8023,10 @@
       <c r="L317" s="9" t="n"/>
       <c r="M317" s="9" t="n"/>
       <c r="N317" s="11" t="n"/>
+      <c r="O317" s="11">
+        <f>IF(D317="","",IF(COUNTIFS($A$5:$A$404,A317,$D$5:$D$404,D317,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A317,$D$5:$D$404,D317,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="11" t="n"/>
@@ -6788,6 +8046,10 @@
       <c r="L318" s="9" t="n"/>
       <c r="M318" s="9" t="n"/>
       <c r="N318" s="11" t="n"/>
+      <c r="O318" s="11">
+        <f>IF(D318="","",IF(COUNTIFS($A$5:$A$404,A318,$D$5:$D$404,D318,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A318,$D$5:$D$404,D318,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="11" t="n"/>
@@ -6807,6 +8069,10 @@
       <c r="L319" s="9" t="n"/>
       <c r="M319" s="9" t="n"/>
       <c r="N319" s="11" t="n"/>
+      <c r="O319" s="11">
+        <f>IF(D319="","",IF(COUNTIFS($A$5:$A$404,A319,$D$5:$D$404,D319,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A319,$D$5:$D$404,D319,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="11" t="n"/>
@@ -6826,6 +8092,10 @@
       <c r="L320" s="9" t="n"/>
       <c r="M320" s="9" t="n"/>
       <c r="N320" s="11" t="n"/>
+      <c r="O320" s="11">
+        <f>IF(D320="","",IF(COUNTIFS($A$5:$A$404,A320,$D$5:$D$404,D320,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A320,$D$5:$D$404,D320,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="11" t="n"/>
@@ -6845,6 +8115,10 @@
       <c r="L321" s="9" t="n"/>
       <c r="M321" s="9" t="n"/>
       <c r="N321" s="11" t="n"/>
+      <c r="O321" s="11">
+        <f>IF(D321="","",IF(COUNTIFS($A$5:$A$404,A321,$D$5:$D$404,D321,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A321,$D$5:$D$404,D321,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="11" t="n"/>
@@ -6864,6 +8138,10 @@
       <c r="L322" s="9" t="n"/>
       <c r="M322" s="9" t="n"/>
       <c r="N322" s="11" t="n"/>
+      <c r="O322" s="11">
+        <f>IF(D322="","",IF(COUNTIFS($A$5:$A$404,A322,$D$5:$D$404,D322,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A322,$D$5:$D$404,D322,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="11" t="n"/>
@@ -6883,6 +8161,10 @@
       <c r="L323" s="9" t="n"/>
       <c r="M323" s="9" t="n"/>
       <c r="N323" s="11" t="n"/>
+      <c r="O323" s="11">
+        <f>IF(D323="","",IF(COUNTIFS($A$5:$A$404,A323,$D$5:$D$404,D323,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A323,$D$5:$D$404,D323,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="11" t="n"/>
@@ -6902,6 +8184,10 @@
       <c r="L324" s="9" t="n"/>
       <c r="M324" s="9" t="n"/>
       <c r="N324" s="11" t="n"/>
+      <c r="O324" s="11">
+        <f>IF(D324="","",IF(COUNTIFS($A$5:$A$404,A324,$D$5:$D$404,D324,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A324,$D$5:$D$404,D324,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="11" t="n"/>
@@ -6921,6 +8207,10 @@
       <c r="L325" s="9" t="n"/>
       <c r="M325" s="9" t="n"/>
       <c r="N325" s="11" t="n"/>
+      <c r="O325" s="11">
+        <f>IF(D325="","",IF(COUNTIFS($A$5:$A$404,A325,$D$5:$D$404,D325,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A325,$D$5:$D$404,D325,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="11" t="n"/>
@@ -6940,6 +8230,10 @@
       <c r="L326" s="9" t="n"/>
       <c r="M326" s="9" t="n"/>
       <c r="N326" s="11" t="n"/>
+      <c r="O326" s="11">
+        <f>IF(D326="","",IF(COUNTIFS($A$5:$A$404,A326,$D$5:$D$404,D326,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A326,$D$5:$D$404,D326,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="11" t="n"/>
@@ -6959,6 +8253,10 @@
       <c r="L327" s="9" t="n"/>
       <c r="M327" s="9" t="n"/>
       <c r="N327" s="11" t="n"/>
+      <c r="O327" s="11">
+        <f>IF(D327="","",IF(COUNTIFS($A$5:$A$404,A327,$D$5:$D$404,D327,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A327,$D$5:$D$404,D327,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="11" t="n"/>
@@ -6978,6 +8276,10 @@
       <c r="L328" s="9" t="n"/>
       <c r="M328" s="9" t="n"/>
       <c r="N328" s="11" t="n"/>
+      <c r="O328" s="11">
+        <f>IF(D328="","",IF(COUNTIFS($A$5:$A$404,A328,$D$5:$D$404,D328,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A328,$D$5:$D$404,D328,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="11" t="n"/>
@@ -6997,6 +8299,10 @@
       <c r="L329" s="9" t="n"/>
       <c r="M329" s="9" t="n"/>
       <c r="N329" s="11" t="n"/>
+      <c r="O329" s="11">
+        <f>IF(D329="","",IF(COUNTIFS($A$5:$A$404,A329,$D$5:$D$404,D329,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A329,$D$5:$D$404,D329,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="11" t="n"/>
@@ -7016,6 +8322,10 @@
       <c r="L330" s="9" t="n"/>
       <c r="M330" s="9" t="n"/>
       <c r="N330" s="11" t="n"/>
+      <c r="O330" s="11">
+        <f>IF(D330="","",IF(COUNTIFS($A$5:$A$404,A330,$D$5:$D$404,D330,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A330,$D$5:$D$404,D330,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="11" t="n"/>
@@ -7035,6 +8345,10 @@
       <c r="L331" s="9" t="n"/>
       <c r="M331" s="9" t="n"/>
       <c r="N331" s="11" t="n"/>
+      <c r="O331" s="11">
+        <f>IF(D331="","",IF(COUNTIFS($A$5:$A$404,A331,$D$5:$D$404,D331,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A331,$D$5:$D$404,D331,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="11" t="n"/>
@@ -7054,6 +8368,10 @@
       <c r="L332" s="9" t="n"/>
       <c r="M332" s="9" t="n"/>
       <c r="N332" s="11" t="n"/>
+      <c r="O332" s="11">
+        <f>IF(D332="","",IF(COUNTIFS($A$5:$A$404,A332,$D$5:$D$404,D332,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A332,$D$5:$D$404,D332,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="11" t="n"/>
@@ -7073,6 +8391,10 @@
       <c r="L333" s="9" t="n"/>
       <c r="M333" s="9" t="n"/>
       <c r="N333" s="11" t="n"/>
+      <c r="O333" s="11">
+        <f>IF(D333="","",IF(COUNTIFS($A$5:$A$404,A333,$D$5:$D$404,D333,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A333,$D$5:$D$404,D333,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="11" t="n"/>
@@ -7092,6 +8414,10 @@
       <c r="L334" s="9" t="n"/>
       <c r="M334" s="9" t="n"/>
       <c r="N334" s="11" t="n"/>
+      <c r="O334" s="11">
+        <f>IF(D334="","",IF(COUNTIFS($A$5:$A$404,A334,$D$5:$D$404,D334,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A334,$D$5:$D$404,D334,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="11" t="n"/>
@@ -7111,6 +8437,10 @@
       <c r="L335" s="9" t="n"/>
       <c r="M335" s="9" t="n"/>
       <c r="N335" s="11" t="n"/>
+      <c r="O335" s="11">
+        <f>IF(D335="","",IF(COUNTIFS($A$5:$A$404,A335,$D$5:$D$404,D335,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A335,$D$5:$D$404,D335,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="11" t="n"/>
@@ -7130,6 +8460,10 @@
       <c r="L336" s="9" t="n"/>
       <c r="M336" s="9" t="n"/>
       <c r="N336" s="11" t="n"/>
+      <c r="O336" s="11">
+        <f>IF(D336="","",IF(COUNTIFS($A$5:$A$404,A336,$D$5:$D$404,D336,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A336,$D$5:$D$404,D336,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="11" t="n"/>
@@ -7149,6 +8483,10 @@
       <c r="L337" s="9" t="n"/>
       <c r="M337" s="9" t="n"/>
       <c r="N337" s="11" t="n"/>
+      <c r="O337" s="11">
+        <f>IF(D337="","",IF(COUNTIFS($A$5:$A$404,A337,$D$5:$D$404,D337,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A337,$D$5:$D$404,D337,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="11" t="n"/>
@@ -7168,6 +8506,10 @@
       <c r="L338" s="9" t="n"/>
       <c r="M338" s="9" t="n"/>
       <c r="N338" s="11" t="n"/>
+      <c r="O338" s="11">
+        <f>IF(D338="","",IF(COUNTIFS($A$5:$A$404,A338,$D$5:$D$404,D338,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A338,$D$5:$D$404,D338,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="11" t="n"/>
@@ -7187,6 +8529,10 @@
       <c r="L339" s="9" t="n"/>
       <c r="M339" s="9" t="n"/>
       <c r="N339" s="11" t="n"/>
+      <c r="O339" s="11">
+        <f>IF(D339="","",IF(COUNTIFS($A$5:$A$404,A339,$D$5:$D$404,D339,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A339,$D$5:$D$404,D339,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="11" t="n"/>
@@ -7206,6 +8552,10 @@
       <c r="L340" s="9" t="n"/>
       <c r="M340" s="9" t="n"/>
       <c r="N340" s="11" t="n"/>
+      <c r="O340" s="11">
+        <f>IF(D340="","",IF(COUNTIFS($A$5:$A$404,A340,$D$5:$D$404,D340,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A340,$D$5:$D$404,D340,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="11" t="n"/>
@@ -7225,6 +8575,10 @@
       <c r="L341" s="9" t="n"/>
       <c r="M341" s="9" t="n"/>
       <c r="N341" s="11" t="n"/>
+      <c r="O341" s="11">
+        <f>IF(D341="","",IF(COUNTIFS($A$5:$A$404,A341,$D$5:$D$404,D341,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A341,$D$5:$D$404,D341,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="11" t="n"/>
@@ -7244,6 +8598,10 @@
       <c r="L342" s="9" t="n"/>
       <c r="M342" s="9" t="n"/>
       <c r="N342" s="11" t="n"/>
+      <c r="O342" s="11">
+        <f>IF(D342="","",IF(COUNTIFS($A$5:$A$404,A342,$D$5:$D$404,D342,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A342,$D$5:$D$404,D342,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="11" t="n"/>
@@ -7263,6 +8621,10 @@
       <c r="L343" s="9" t="n"/>
       <c r="M343" s="9" t="n"/>
       <c r="N343" s="11" t="n"/>
+      <c r="O343" s="11">
+        <f>IF(D343="","",IF(COUNTIFS($A$5:$A$404,A343,$D$5:$D$404,D343,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A343,$D$5:$D$404,D343,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="11" t="n"/>
@@ -7282,6 +8644,10 @@
       <c r="L344" s="9" t="n"/>
       <c r="M344" s="9" t="n"/>
       <c r="N344" s="11" t="n"/>
+      <c r="O344" s="11">
+        <f>IF(D344="","",IF(COUNTIFS($A$5:$A$404,A344,$D$5:$D$404,D344,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A344,$D$5:$D$404,D344,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="11" t="n"/>
@@ -7301,6 +8667,10 @@
       <c r="L345" s="9" t="n"/>
       <c r="M345" s="9" t="n"/>
       <c r="N345" s="11" t="n"/>
+      <c r="O345" s="11">
+        <f>IF(D345="","",IF(COUNTIFS($A$5:$A$404,A345,$D$5:$D$404,D345,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A345,$D$5:$D$404,D345,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="11" t="n"/>
@@ -7320,6 +8690,10 @@
       <c r="L346" s="9" t="n"/>
       <c r="M346" s="9" t="n"/>
       <c r="N346" s="11" t="n"/>
+      <c r="O346" s="11">
+        <f>IF(D346="","",IF(COUNTIFS($A$5:$A$404,A346,$D$5:$D$404,D346,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A346,$D$5:$D$404,D346,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="11" t="n"/>
@@ -7339,6 +8713,10 @@
       <c r="L347" s="9" t="n"/>
       <c r="M347" s="9" t="n"/>
       <c r="N347" s="11" t="n"/>
+      <c r="O347" s="11">
+        <f>IF(D347="","",IF(COUNTIFS($A$5:$A$404,A347,$D$5:$D$404,D347,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A347,$D$5:$D$404,D347,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="11" t="n"/>
@@ -7358,6 +8736,10 @@
       <c r="L348" s="9" t="n"/>
       <c r="M348" s="9" t="n"/>
       <c r="N348" s="11" t="n"/>
+      <c r="O348" s="11">
+        <f>IF(D348="","",IF(COUNTIFS($A$5:$A$404,A348,$D$5:$D$404,D348,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A348,$D$5:$D$404,D348,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="11" t="n"/>
@@ -7377,6 +8759,10 @@
       <c r="L349" s="9" t="n"/>
       <c r="M349" s="9" t="n"/>
       <c r="N349" s="11" t="n"/>
+      <c r="O349" s="11">
+        <f>IF(D349="","",IF(COUNTIFS($A$5:$A$404,A349,$D$5:$D$404,D349,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A349,$D$5:$D$404,D349,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="11" t="n"/>
@@ -7396,6 +8782,10 @@
       <c r="L350" s="9" t="n"/>
       <c r="M350" s="9" t="n"/>
       <c r="N350" s="11" t="n"/>
+      <c r="O350" s="11">
+        <f>IF(D350="","",IF(COUNTIFS($A$5:$A$404,A350,$D$5:$D$404,D350,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A350,$D$5:$D$404,D350,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="11" t="n"/>
@@ -7415,6 +8805,10 @@
       <c r="L351" s="9" t="n"/>
       <c r="M351" s="9" t="n"/>
       <c r="N351" s="11" t="n"/>
+      <c r="O351" s="11">
+        <f>IF(D351="","",IF(COUNTIFS($A$5:$A$404,A351,$D$5:$D$404,D351,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A351,$D$5:$D$404,D351,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="11" t="n"/>
@@ -7434,6 +8828,10 @@
       <c r="L352" s="9" t="n"/>
       <c r="M352" s="9" t="n"/>
       <c r="N352" s="11" t="n"/>
+      <c r="O352" s="11">
+        <f>IF(D352="","",IF(COUNTIFS($A$5:$A$404,A352,$D$5:$D$404,D352,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A352,$D$5:$D$404,D352,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="353">
       <c r="A353" s="11" t="n"/>
@@ -7453,6 +8851,10 @@
       <c r="L353" s="9" t="n"/>
       <c r="M353" s="9" t="n"/>
       <c r="N353" s="11" t="n"/>
+      <c r="O353" s="11">
+        <f>IF(D353="","",IF(COUNTIFS($A$5:$A$404,A353,$D$5:$D$404,D353,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A353,$D$5:$D$404,D353,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="11" t="n"/>
@@ -7472,6 +8874,10 @@
       <c r="L354" s="9" t="n"/>
       <c r="M354" s="9" t="n"/>
       <c r="N354" s="11" t="n"/>
+      <c r="O354" s="11">
+        <f>IF(D354="","",IF(COUNTIFS($A$5:$A$404,A354,$D$5:$D$404,D354,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A354,$D$5:$D$404,D354,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="11" t="n"/>
@@ -7491,6 +8897,10 @@
       <c r="L355" s="9" t="n"/>
       <c r="M355" s="9" t="n"/>
       <c r="N355" s="11" t="n"/>
+      <c r="O355" s="11">
+        <f>IF(D355="","",IF(COUNTIFS($A$5:$A$404,A355,$D$5:$D$404,D355,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A355,$D$5:$D$404,D355,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="11" t="n"/>
@@ -7510,6 +8920,10 @@
       <c r="L356" s="9" t="n"/>
       <c r="M356" s="9" t="n"/>
       <c r="N356" s="11" t="n"/>
+      <c r="O356" s="11">
+        <f>IF(D356="","",IF(COUNTIFS($A$5:$A$404,A356,$D$5:$D$404,D356,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A356,$D$5:$D$404,D356,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="11" t="n"/>
@@ -7529,6 +8943,10 @@
       <c r="L357" s="9" t="n"/>
       <c r="M357" s="9" t="n"/>
       <c r="N357" s="11" t="n"/>
+      <c r="O357" s="11">
+        <f>IF(D357="","",IF(COUNTIFS($A$5:$A$404,A357,$D$5:$D$404,D357,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A357,$D$5:$D$404,D357,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="11" t="n"/>
@@ -7548,6 +8966,10 @@
       <c r="L358" s="9" t="n"/>
       <c r="M358" s="9" t="n"/>
       <c r="N358" s="11" t="n"/>
+      <c r="O358" s="11">
+        <f>IF(D358="","",IF(COUNTIFS($A$5:$A$404,A358,$D$5:$D$404,D358,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A358,$D$5:$D$404,D358,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="11" t="n"/>
@@ -7567,6 +8989,10 @@
       <c r="L359" s="9" t="n"/>
       <c r="M359" s="9" t="n"/>
       <c r="N359" s="11" t="n"/>
+      <c r="O359" s="11">
+        <f>IF(D359="","",IF(COUNTIFS($A$5:$A$404,A359,$D$5:$D$404,D359,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A359,$D$5:$D$404,D359,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="11" t="n"/>
@@ -7586,6 +9012,10 @@
       <c r="L360" s="9" t="n"/>
       <c r="M360" s="9" t="n"/>
       <c r="N360" s="11" t="n"/>
+      <c r="O360" s="11">
+        <f>IF(D360="","",IF(COUNTIFS($A$5:$A$404,A360,$D$5:$D$404,D360,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A360,$D$5:$D$404,D360,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="11" t="n"/>
@@ -7605,6 +9035,10 @@
       <c r="L361" s="9" t="n"/>
       <c r="M361" s="9" t="n"/>
       <c r="N361" s="11" t="n"/>
+      <c r="O361" s="11">
+        <f>IF(D361="","",IF(COUNTIFS($A$5:$A$404,A361,$D$5:$D$404,D361,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A361,$D$5:$D$404,D361,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="11" t="n"/>
@@ -7624,6 +9058,10 @@
       <c r="L362" s="9" t="n"/>
       <c r="M362" s="9" t="n"/>
       <c r="N362" s="11" t="n"/>
+      <c r="O362" s="11">
+        <f>IF(D362="","",IF(COUNTIFS($A$5:$A$404,A362,$D$5:$D$404,D362,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A362,$D$5:$D$404,D362,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="11" t="n"/>
@@ -7643,6 +9081,10 @@
       <c r="L363" s="9" t="n"/>
       <c r="M363" s="9" t="n"/>
       <c r="N363" s="11" t="n"/>
+      <c r="O363" s="11">
+        <f>IF(D363="","",IF(COUNTIFS($A$5:$A$404,A363,$D$5:$D$404,D363,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A363,$D$5:$D$404,D363,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="11" t="n"/>
@@ -7662,6 +9104,10 @@
       <c r="L364" s="9" t="n"/>
       <c r="M364" s="9" t="n"/>
       <c r="N364" s="11" t="n"/>
+      <c r="O364" s="11">
+        <f>IF(D364="","",IF(COUNTIFS($A$5:$A$404,A364,$D$5:$D$404,D364,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A364,$D$5:$D$404,D364,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="11" t="n"/>
@@ -7681,6 +9127,10 @@
       <c r="L365" s="9" t="n"/>
       <c r="M365" s="9" t="n"/>
       <c r="N365" s="11" t="n"/>
+      <c r="O365" s="11">
+        <f>IF(D365="","",IF(COUNTIFS($A$5:$A$404,A365,$D$5:$D$404,D365,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A365,$D$5:$D$404,D365,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="11" t="n"/>
@@ -7700,6 +9150,10 @@
       <c r="L366" s="9" t="n"/>
       <c r="M366" s="9" t="n"/>
       <c r="N366" s="11" t="n"/>
+      <c r="O366" s="11">
+        <f>IF(D366="","",IF(COUNTIFS($A$5:$A$404,A366,$D$5:$D$404,D366,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A366,$D$5:$D$404,D366,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="11" t="n"/>
@@ -7719,6 +9173,10 @@
       <c r="L367" s="9" t="n"/>
       <c r="M367" s="9" t="n"/>
       <c r="N367" s="11" t="n"/>
+      <c r="O367" s="11">
+        <f>IF(D367="","",IF(COUNTIFS($A$5:$A$404,A367,$D$5:$D$404,D367,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A367,$D$5:$D$404,D367,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="11" t="n"/>
@@ -7738,6 +9196,10 @@
       <c r="L368" s="9" t="n"/>
       <c r="M368" s="9" t="n"/>
       <c r="N368" s="11" t="n"/>
+      <c r="O368" s="11">
+        <f>IF(D368="","",IF(COUNTIFS($A$5:$A$404,A368,$D$5:$D$404,D368,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A368,$D$5:$D$404,D368,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="11" t="n"/>
@@ -7757,6 +9219,10 @@
       <c r="L369" s="9" t="n"/>
       <c r="M369" s="9" t="n"/>
       <c r="N369" s="11" t="n"/>
+      <c r="O369" s="11">
+        <f>IF(D369="","",IF(COUNTIFS($A$5:$A$404,A369,$D$5:$D$404,D369,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A369,$D$5:$D$404,D369,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="11" t="n"/>
@@ -7776,6 +9242,10 @@
       <c r="L370" s="9" t="n"/>
       <c r="M370" s="9" t="n"/>
       <c r="N370" s="11" t="n"/>
+      <c r="O370" s="11">
+        <f>IF(D370="","",IF(COUNTIFS($A$5:$A$404,A370,$D$5:$D$404,D370,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A370,$D$5:$D$404,D370,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="11" t="n"/>
@@ -7795,6 +9265,10 @@
       <c r="L371" s="9" t="n"/>
       <c r="M371" s="9" t="n"/>
       <c r="N371" s="11" t="n"/>
+      <c r="O371" s="11">
+        <f>IF(D371="","",IF(COUNTIFS($A$5:$A$404,A371,$D$5:$D$404,D371,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A371,$D$5:$D$404,D371,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="11" t="n"/>
@@ -7814,6 +9288,10 @@
       <c r="L372" s="9" t="n"/>
       <c r="M372" s="9" t="n"/>
       <c r="N372" s="11" t="n"/>
+      <c r="O372" s="11">
+        <f>IF(D372="","",IF(COUNTIFS($A$5:$A$404,A372,$D$5:$D$404,D372,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A372,$D$5:$D$404,D372,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="11" t="n"/>
@@ -7833,6 +9311,10 @@
       <c r="L373" s="9" t="n"/>
       <c r="M373" s="9" t="n"/>
       <c r="N373" s="11" t="n"/>
+      <c r="O373" s="11">
+        <f>IF(D373="","",IF(COUNTIFS($A$5:$A$404,A373,$D$5:$D$404,D373,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A373,$D$5:$D$404,D373,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="11" t="n"/>
@@ -7852,6 +9334,10 @@
       <c r="L374" s="9" t="n"/>
       <c r="M374" s="9" t="n"/>
       <c r="N374" s="11" t="n"/>
+      <c r="O374" s="11">
+        <f>IF(D374="","",IF(COUNTIFS($A$5:$A$404,A374,$D$5:$D$404,D374,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A374,$D$5:$D$404,D374,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="11" t="n"/>
@@ -7871,6 +9357,10 @@
       <c r="L375" s="9" t="n"/>
       <c r="M375" s="9" t="n"/>
       <c r="N375" s="11" t="n"/>
+      <c r="O375" s="11">
+        <f>IF(D375="","",IF(COUNTIFS($A$5:$A$404,A375,$D$5:$D$404,D375,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A375,$D$5:$D$404,D375,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="11" t="n"/>
@@ -7890,6 +9380,10 @@
       <c r="L376" s="9" t="n"/>
       <c r="M376" s="9" t="n"/>
       <c r="N376" s="11" t="n"/>
+      <c r="O376" s="11">
+        <f>IF(D376="","",IF(COUNTIFS($A$5:$A$404,A376,$D$5:$D$404,D376,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A376,$D$5:$D$404,D376,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="11" t="n"/>
@@ -7909,6 +9403,10 @@
       <c r="L377" s="9" t="n"/>
       <c r="M377" s="9" t="n"/>
       <c r="N377" s="11" t="n"/>
+      <c r="O377" s="11">
+        <f>IF(D377="","",IF(COUNTIFS($A$5:$A$404,A377,$D$5:$D$404,D377,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A377,$D$5:$D$404,D377,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="11" t="n"/>
@@ -7928,6 +9426,10 @@
       <c r="L378" s="9" t="n"/>
       <c r="M378" s="9" t="n"/>
       <c r="N378" s="11" t="n"/>
+      <c r="O378" s="11">
+        <f>IF(D378="","",IF(COUNTIFS($A$5:$A$404,A378,$D$5:$D$404,D378,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A378,$D$5:$D$404,D378,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="11" t="n"/>
@@ -7947,6 +9449,10 @@
       <c r="L379" s="9" t="n"/>
       <c r="M379" s="9" t="n"/>
       <c r="N379" s="11" t="n"/>
+      <c r="O379" s="11">
+        <f>IF(D379="","",IF(COUNTIFS($A$5:$A$404,A379,$D$5:$D$404,D379,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A379,$D$5:$D$404,D379,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="11" t="n"/>
@@ -7966,6 +9472,10 @@
       <c r="L380" s="9" t="n"/>
       <c r="M380" s="9" t="n"/>
       <c r="N380" s="11" t="n"/>
+      <c r="O380" s="11">
+        <f>IF(D380="","",IF(COUNTIFS($A$5:$A$404,A380,$D$5:$D$404,D380,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A380,$D$5:$D$404,D380,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="11" t="n"/>
@@ -7985,6 +9495,10 @@
       <c r="L381" s="9" t="n"/>
       <c r="M381" s="9" t="n"/>
       <c r="N381" s="11" t="n"/>
+      <c r="O381" s="11">
+        <f>IF(D381="","",IF(COUNTIFS($A$5:$A$404,A381,$D$5:$D$404,D381,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A381,$D$5:$D$404,D381,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="382">
       <c r="A382" s="11" t="n"/>
@@ -8004,6 +9518,10 @@
       <c r="L382" s="9" t="n"/>
       <c r="M382" s="9" t="n"/>
       <c r="N382" s="11" t="n"/>
+      <c r="O382" s="11">
+        <f>IF(D382="","",IF(COUNTIFS($A$5:$A$404,A382,$D$5:$D$404,D382,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A382,$D$5:$D$404,D382,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="11" t="n"/>
@@ -8023,6 +9541,10 @@
       <c r="L383" s="9" t="n"/>
       <c r="M383" s="9" t="n"/>
       <c r="N383" s="11" t="n"/>
+      <c r="O383" s="11">
+        <f>IF(D383="","",IF(COUNTIFS($A$5:$A$404,A383,$D$5:$D$404,D383,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A383,$D$5:$D$404,D383,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="384">
       <c r="A384" s="11" t="n"/>
@@ -8042,6 +9564,10 @@
       <c r="L384" s="9" t="n"/>
       <c r="M384" s="9" t="n"/>
       <c r="N384" s="11" t="n"/>
+      <c r="O384" s="11">
+        <f>IF(D384="","",IF(COUNTIFS($A$5:$A$404,A384,$D$5:$D$404,D384,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A384,$D$5:$D$404,D384,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="11" t="n"/>
@@ -8061,6 +9587,10 @@
       <c r="L385" s="9" t="n"/>
       <c r="M385" s="9" t="n"/>
       <c r="N385" s="11" t="n"/>
+      <c r="O385" s="11">
+        <f>IF(D385="","",IF(COUNTIFS($A$5:$A$404,A385,$D$5:$D$404,D385,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A385,$D$5:$D$404,D385,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="386">
       <c r="A386" s="11" t="n"/>
@@ -8080,6 +9610,10 @@
       <c r="L386" s="9" t="n"/>
       <c r="M386" s="9" t="n"/>
       <c r="N386" s="11" t="n"/>
+      <c r="O386" s="11">
+        <f>IF(D386="","",IF(COUNTIFS($A$5:$A$404,A386,$D$5:$D$404,D386,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A386,$D$5:$D$404,D386,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="387">
       <c r="A387" s="11" t="n"/>
@@ -8099,6 +9633,10 @@
       <c r="L387" s="9" t="n"/>
       <c r="M387" s="9" t="n"/>
       <c r="N387" s="11" t="n"/>
+      <c r="O387" s="11">
+        <f>IF(D387="","",IF(COUNTIFS($A$5:$A$404,A387,$D$5:$D$404,D387,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A387,$D$5:$D$404,D387,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="11" t="n"/>
@@ -8118,6 +9656,10 @@
       <c r="L388" s="9" t="n"/>
       <c r="M388" s="9" t="n"/>
       <c r="N388" s="11" t="n"/>
+      <c r="O388" s="11">
+        <f>IF(D388="","",IF(COUNTIFS($A$5:$A$404,A388,$D$5:$D$404,D388,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A388,$D$5:$D$404,D388,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="389">
       <c r="A389" s="11" t="n"/>
@@ -8137,6 +9679,10 @@
       <c r="L389" s="9" t="n"/>
       <c r="M389" s="9" t="n"/>
       <c r="N389" s="11" t="n"/>
+      <c r="O389" s="11">
+        <f>IF(D389="","",IF(COUNTIFS($A$5:$A$404,A389,$D$5:$D$404,D389,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A389,$D$5:$D$404,D389,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="390">
       <c r="A390" s="11" t="n"/>
@@ -8156,6 +9702,10 @@
       <c r="L390" s="9" t="n"/>
       <c r="M390" s="9" t="n"/>
       <c r="N390" s="11" t="n"/>
+      <c r="O390" s="11">
+        <f>IF(D390="","",IF(COUNTIFS($A$5:$A$404,A390,$D$5:$D$404,D390,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A390,$D$5:$D$404,D390,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="391">
       <c r="A391" s="11" t="n"/>
@@ -8175,6 +9725,10 @@
       <c r="L391" s="9" t="n"/>
       <c r="M391" s="9" t="n"/>
       <c r="N391" s="11" t="n"/>
+      <c r="O391" s="11">
+        <f>IF(D391="","",IF(COUNTIFS($A$5:$A$404,A391,$D$5:$D$404,D391,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A391,$D$5:$D$404,D391,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="392">
       <c r="A392" s="11" t="n"/>
@@ -8194,6 +9748,10 @@
       <c r="L392" s="9" t="n"/>
       <c r="M392" s="9" t="n"/>
       <c r="N392" s="11" t="n"/>
+      <c r="O392" s="11">
+        <f>IF(D392="","",IF(COUNTIFS($A$5:$A$404,A392,$D$5:$D$404,D392,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A392,$D$5:$D$404,D392,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="393">
       <c r="A393" s="11" t="n"/>
@@ -8213,6 +9771,10 @@
       <c r="L393" s="9" t="n"/>
       <c r="M393" s="9" t="n"/>
       <c r="N393" s="11" t="n"/>
+      <c r="O393" s="11">
+        <f>IF(D393="","",IF(COUNTIFS($A$5:$A$404,A393,$D$5:$D$404,D393,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A393,$D$5:$D$404,D393,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="394">
       <c r="A394" s="11" t="n"/>
@@ -8232,6 +9794,10 @@
       <c r="L394" s="9" t="n"/>
       <c r="M394" s="9" t="n"/>
       <c r="N394" s="11" t="n"/>
+      <c r="O394" s="11">
+        <f>IF(D394="","",IF(COUNTIFS($A$5:$A$404,A394,$D$5:$D$404,D394,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A394,$D$5:$D$404,D394,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="395">
       <c r="A395" s="11" t="n"/>
@@ -8251,6 +9817,10 @@
       <c r="L395" s="9" t="n"/>
       <c r="M395" s="9" t="n"/>
       <c r="N395" s="11" t="n"/>
+      <c r="O395" s="11">
+        <f>IF(D395="","",IF(COUNTIFS($A$5:$A$404,A395,$D$5:$D$404,D395,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A395,$D$5:$D$404,D395,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="396">
       <c r="A396" s="11" t="n"/>
@@ -8270,6 +9840,10 @@
       <c r="L396" s="9" t="n"/>
       <c r="M396" s="9" t="n"/>
       <c r="N396" s="11" t="n"/>
+      <c r="O396" s="11">
+        <f>IF(D396="","",IF(COUNTIFS($A$5:$A$404,A396,$D$5:$D$404,D396,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A396,$D$5:$D$404,D396,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="397">
       <c r="A397" s="11" t="n"/>
@@ -8289,6 +9863,10 @@
       <c r="L397" s="9" t="n"/>
       <c r="M397" s="9" t="n"/>
       <c r="N397" s="11" t="n"/>
+      <c r="O397" s="11">
+        <f>IF(D397="","",IF(COUNTIFS($A$5:$A$404,A397,$D$5:$D$404,D397,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A397,$D$5:$D$404,D397,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="11" t="n"/>
@@ -8308,6 +9886,10 @@
       <c r="L398" s="9" t="n"/>
       <c r="M398" s="9" t="n"/>
       <c r="N398" s="11" t="n"/>
+      <c r="O398" s="11">
+        <f>IF(D398="","",IF(COUNTIFS($A$5:$A$404,A398,$D$5:$D$404,D398,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A398,$D$5:$D$404,D398,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="399">
       <c r="A399" s="11" t="n"/>
@@ -8327,6 +9909,10 @@
       <c r="L399" s="9" t="n"/>
       <c r="M399" s="9" t="n"/>
       <c r="N399" s="11" t="n"/>
+      <c r="O399" s="11">
+        <f>IF(D399="","",IF(COUNTIFS($A$5:$A$404,A399,$D$5:$D$404,D399,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A399,$D$5:$D$404,D399,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="400">
       <c r="A400" s="11" t="n"/>
@@ -8346,6 +9932,10 @@
       <c r="L400" s="9" t="n"/>
       <c r="M400" s="9" t="n"/>
       <c r="N400" s="11" t="n"/>
+      <c r="O400" s="11">
+        <f>IF(D400="","",IF(COUNTIFS($A$5:$A$404,A400,$D$5:$D$404,D400,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A400,$D$5:$D$404,D400,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="11" t="n"/>
@@ -8365,6 +9955,10 @@
       <c r="L401" s="9" t="n"/>
       <c r="M401" s="9" t="n"/>
       <c r="N401" s="11" t="n"/>
+      <c r="O401" s="11">
+        <f>IF(D401="","",IF(COUNTIFS($A$5:$A$404,A401,$D$5:$D$404,D401,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A401,$D$5:$D$404,D401,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="402">
       <c r="A402" s="11" t="n"/>
@@ -8384,6 +9978,10 @@
       <c r="L402" s="9" t="n"/>
       <c r="M402" s="9" t="n"/>
       <c r="N402" s="11" t="n"/>
+      <c r="O402" s="11">
+        <f>IF(D402="","",IF(COUNTIFS($A$5:$A$404,A402,$D$5:$D$404,D402,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A402,$D$5:$D$404,D402,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="403">
       <c r="A403" s="11" t="n"/>
@@ -8403,6 +10001,10 @@
       <c r="L403" s="9" t="n"/>
       <c r="M403" s="9" t="n"/>
       <c r="N403" s="11" t="n"/>
+      <c r="O403" s="11">
+        <f>IF(D403="","",IF(COUNTIFS($A$5:$A$404,A403,$D$5:$D$404,D403,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A403,$D$5:$D$404,D403,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
     <row r="404">
       <c r="A404" s="11" t="n"/>
@@ -8422,9 +10024,13 @@
       <c r="L404" s="9" t="n"/>
       <c r="M404" s="9" t="n"/>
       <c r="N404" s="11" t="n"/>
+      <c r="O404" s="11">
+        <f>IF(D404="","",IF(COUNTIFS($A$5:$A$404,A404,$D$5:$D$404,D404,$I$5:$I$404,"ja")=4,"compleet",COUNTIFS($A$5:$A$404,A404,$D$5:$D$404,D404,$I$5:$I$404,"ja")&amp;" van 4"))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N404"/>
+  <autoFilter ref="A4:O404"/>
   <conditionalFormatting sqref="J5:K404">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND($H5="ja",$J5="nee")</formula>
@@ -8433,6 +10039,11 @@
   <conditionalFormatting sqref="I5:I404">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>$I5="ja"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O5:O404">
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>$O5="compleet"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
@@ -8460,7 +10071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -8500,64 +10111,71 @@
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>3. Zet per speler Aanwezig op "ja".</t>
+          <t>3. Zet per speler Aanwezig op "ja". Kolom Groep compleet laat zien of alle vier er zijn ("compleet" of bijvoorbeeld "3 van 4").</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>4. Kijk per speler: echt verkleed of geschminkt? Zet Echt verkleed? op "ja" of "nee".</t>
+          <t xml:space="preserve">   Nog niet compleet? Laat ze wachten tot de vierde er is, uiterlijk tot de begintijd. Pas als de groep compleet is, gaan ze naar de baan.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Telt WEL: volledig kostuum, schmink of facepaint over het hele gezicht, masker met kostuum.</t>
+          <t>4. Kijk per speler: echt verkleed of geschminkt? Zet Echt verkleed? op "ja" of "nee".</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Telt NIET: alleen een hoedje of oortjes, een gewoon shirt met print, twee streepjes schmink.</t>
+          <t xml:space="preserve">   Telt WEL: volledig kostuum, schmink of facepaint over het hele gezicht, masker met kostuum.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>5. Wordt de cel oranje? Dan heeft die speler korting betaald maar is hij of zij niet echt verkleed.</t>
+          <t xml:space="preserve">   Telt NIET: alleen een hoedje of oortjes, een gewoon shirt met print, twee streepjes schmink.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Bij te betalen staat in kolom K (1 uur: €4,69 · 1,5 uur: €7,03 · 2 uur: €9,38). Laat dat ter plekke bijbetalen en vul Bijbetaald via in.</t>
+          <t>5. Wordt de cel oranje? Dan heeft die speler korting betaald maar is hij of zij niet echt verkleed.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>6. Noem het baannummer (kolom Baan) en wens ze een griezelige wedstrijd.</t>
+          <t xml:space="preserve">   Bij te betalen staat in kolom K (1 uur: €4,69 · 1,5 uur: €7,03 · 2 uur: €9,38). Laat dat ter plekke bijbetalen en vul Bijbetaald via in.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr"/>
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>6. Pas nu noem je het baannummer (kolom Baan). De spelers weten dat van tevoren niet. Wens ze een griezelige wedstrijd.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Twijfel over een kostuum? Kies voor de speler, het is een feestje. Mooie outfits: maak een foto voor Instagram (vraag eerst even of het mag).</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Staat iemand niet op de lijst? Kijk in Mollie (Betalingen, zoek op naam) of in Netlify Forms (halloween-boeking). Niet betaald = gewoon tarief via Poort Padel.</t>
         </is>

</xml_diff>

<commit_message>
Halloween terug naar za 31 oktober, 16:00-23:00: site, poster, check-inlijst en teksten
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/events/2026-halloween-padel/checkin/halloween-checkin-lijst.xlsx
+++ b/events/2026-halloween-padel/checkin/halloween-checkin-lijst.xlsx
@@ -551,7 +551,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Halloween Padel Special · check-in · zondag 1 november 2026, 16:00 tot 23:00</t>
+          <t>Halloween Padel Special · check-in · zaterdag 31 oktober 2026, 16:00 tot 23:00</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
@@ -10087,7 +10087,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Zondag 1 november 2026, 16:00 tot 23:00, bij Poort Padel. Spelers komen 10 minuten voor hun begintijd.</t>
+          <t>Zaterdag 31 oktober 2026, 16:00 tot 23:00, bij Poort Padel. Spelers komen 10 minuten voor hun begintijd.</t>
         </is>
       </c>
     </row>

</xml_diff>